<commit_message>
Add internationalization support for English and Hindi languages
- Created common and login JSON files for English translations.
- Created common and login JSON files for Hindi translations.
- Integrated i18next for language support in the main application.
- Updated AdminDashboard, AuditorDashboard, CSODashboard, CitizenDashboard, NodalOfficerDashboard, and Login components to utilize translations.
- Changed references from "Legal Knowledge System" to "Legal Repository" in various components.
- Improved accessibility by adding scope attributes to table headers.
</commit_message>
<xml_diff>
--- a/GIGW_DBIM_Compliance_Tasks.xlsx
+++ b/GIGW_DBIM_Compliance_Tasks.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\TOR PROJECT\hlks-demo\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EA8936B7-8536-4335-AE22-28F5E416FC40}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{045DDB39-22C4-4F9F-88EA-E3E89B0D112B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="580" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Summary" sheetId="1" r:id="rId1"/>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="405" uniqueCount="220">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="412" uniqueCount="221">
   <si>
     <t>GIGW + DBIM Compliance Task Summary</t>
   </si>
@@ -132,6 +132,9 @@
   </si>
   <si>
     <t>File(s) / Area to Touch</t>
+  </si>
+  <si>
+    <t>Status</t>
   </si>
   <si>
     <t>Adopt one official DBIM primary colour group (currently uses a custom blue #1a56db not present in any DBIM palette)</t>
@@ -699,12 +702,18 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF00B050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -719,8 +728,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -784,10 +794,10 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Jpan" typeface="ï¼­ï¼³ ï¼°ã´ã·ãã¯"/>
+        <a:font script="Hang" typeface="ë§ì ê³ ë"/>
+        <a:font script="Hans" typeface="å®ä½"/>
+        <a:font script="Hant" typeface="æ°ç´°æé«"/>
         <a:font script="Arab" typeface="Times New Roman"/>
         <a:font script="Hebr" typeface="Times New Roman"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -819,10 +829,10 @@
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Jpan" typeface="ï¼­ï¼³ ï¼°ã´ã·ãã¯"/>
+        <a:font script="Hang" typeface="ë§ì ê³ ë"/>
+        <a:font script="Hans" typeface="å®ä½"/>
+        <a:font script="Hant" typeface="æ°ç´°æé«"/>
         <a:font script="Arab" typeface="Arial"/>
         <a:font script="Hebr" typeface="Arial"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -1067,12 +1077,12 @@
     <col min="2" max="2" width="50.796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>1</v>
       </c>
@@ -1080,7 +1090,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -1088,7 +1098,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="5" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:2" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>5</v>
       </c>
@@ -1096,7 +1106,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="6" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:2" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>7</v>
       </c>
@@ -1104,7 +1114,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="7" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:2" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>8</v>
       </c>
@@ -1112,7 +1122,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="8" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:2" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>9</v>
       </c>
@@ -1120,7 +1130,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="9" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:2" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>10</v>
       </c>
@@ -1128,7 +1138,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="10" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:2" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>11</v>
       </c>
@@ -1136,7 +1146,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:2" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>12</v>
       </c>
@@ -1144,7 +1154,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:2" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>13</v>
       </c>
@@ -1152,7 +1162,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="14" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:2" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>14</v>
       </c>
@@ -1160,7 +1170,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="15" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:2" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>15</v>
       </c>
@@ -1168,7 +1178,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="16" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:2" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>16</v>
       </c>
@@ -1176,7 +1186,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="17" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:2" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>17</v>
       </c>
@@ -1184,7 +1194,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="18" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:2" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>18</v>
       </c>
@@ -1192,7 +1202,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="19" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:2" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>19</v>
       </c>
@@ -1200,7 +1210,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="20" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:2" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>20</v>
       </c>
@@ -1208,7 +1218,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="21" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:2" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>21</v>
       </c>
@@ -1216,7 +1226,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="22" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:2" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>22</v>
       </c>
@@ -1224,7 +1234,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="23" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:2" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>23</v>
       </c>
@@ -1232,7 +1242,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="24" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:2" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>24</v>
       </c>
@@ -1240,7 +1250,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="25" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:2" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>25</v>
       </c>
@@ -1248,7 +1258,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="27" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:2" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>26</v>
       </c>
@@ -1266,7 +1276,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:I47"/>
+  <dimension ref="A1:J47"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="6.796875" customWidth="1"/>
@@ -1276,10 +1286,10 @@
     <col min="5" max="5" width="16.796875" customWidth="1"/>
     <col min="6" max="6" width="118.59765625" customWidth="1"/>
     <col min="7" max="8" width="10.796875" customWidth="1"/>
-    <col min="9" max="9" width="38.796875" customWidth="1"/>
+    <col min="9" max="9" width="61.09765625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>27</v>
       </c>
@@ -1307,8 +1317,11 @@
       <c r="I1" t="s">
         <v>35</v>
       </c>
-    </row>
-    <row r="2" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="J1" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>1</v>
       </c>
@@ -1316,28 +1329,28 @@
         <v>19</v>
       </c>
       <c r="C2" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D2" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="E2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="F2" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="G2" t="s">
         <v>7</v>
       </c>
       <c r="H2" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="I2" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="3" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>2</v>
       </c>
@@ -1345,28 +1358,28 @@
         <v>19</v>
       </c>
       <c r="C3" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="D3" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="E3" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="F3" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="G3" t="s">
         <v>8</v>
       </c>
       <c r="H3" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="I3" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="4" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>3</v>
       </c>
@@ -1374,28 +1387,28 @@
         <v>19</v>
       </c>
       <c r="C4" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="D4" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="E4" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="F4" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="G4" t="s">
         <v>7</v>
       </c>
       <c r="H4" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="I4" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>4</v>
       </c>
@@ -1403,16 +1416,16 @@
         <v>16</v>
       </c>
       <c r="C5" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="D5" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="E5" t="s">
         <v>11</v>
       </c>
       <c r="F5" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="G5" t="s">
         <v>11</v>
@@ -1421,10 +1434,13 @@
         <v>10</v>
       </c>
       <c r="I5" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="6" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+        <v>55</v>
+      </c>
+      <c r="J5" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>5</v>
       </c>
@@ -1432,28 +1448,28 @@
         <v>16</v>
       </c>
       <c r="C6" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="D6" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="E6" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="F6" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="G6" t="s">
         <v>7</v>
       </c>
       <c r="H6" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="I6" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="7" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>6</v>
       </c>
@@ -1461,28 +1477,28 @@
         <v>16</v>
       </c>
       <c r="C7" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="D7" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="E7" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="F7" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="G7" t="s">
         <v>8</v>
       </c>
       <c r="H7" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="I7" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="8" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>7</v>
       </c>
@@ -1490,28 +1506,28 @@
         <v>16</v>
       </c>
       <c r="C8" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="D8" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="E8" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="F8" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="G8" t="s">
         <v>8</v>
       </c>
       <c r="H8" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="I8" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="9" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>8</v>
       </c>
@@ -1519,28 +1535,28 @@
         <v>16</v>
       </c>
       <c r="C9" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="D9" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E9" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="F9" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="G9" t="s">
         <v>7</v>
       </c>
       <c r="H9" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="I9" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="10" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>9</v>
       </c>
@@ -1548,28 +1564,28 @@
         <v>18</v>
       </c>
       <c r="C10" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="D10" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="E10" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="F10" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="G10" t="s">
         <v>9</v>
       </c>
       <c r="H10" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="I10" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="11" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>10</v>
       </c>
@@ -1577,28 +1593,28 @@
         <v>18</v>
       </c>
       <c r="C11" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="D11" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="E11" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="F11" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="G11" t="s">
         <v>7</v>
       </c>
       <c r="H11" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="I11" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="12" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12">
         <v>11</v>
       </c>
@@ -1606,28 +1622,28 @@
         <v>18</v>
       </c>
       <c r="C12" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="D12" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="E12" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="F12" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="G12" t="s">
         <v>9</v>
       </c>
       <c r="H12" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="I12" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="13" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>12</v>
       </c>
@@ -1635,28 +1651,28 @@
         <v>18</v>
       </c>
       <c r="C13" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="D13" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="E13" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="F13" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="G13" t="s">
         <v>7</v>
       </c>
       <c r="H13" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="I13" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="14" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14">
         <v>13</v>
       </c>
@@ -1664,28 +1680,28 @@
         <v>15</v>
       </c>
       <c r="C14" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="D14" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="E14" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="F14" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="G14" t="s">
         <v>8</v>
       </c>
       <c r="H14" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="I14" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="15" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15">
         <v>14</v>
       </c>
@@ -1693,28 +1709,28 @@
         <v>15</v>
       </c>
       <c r="C15" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="D15" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="E15" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="F15" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="G15" t="s">
         <v>9</v>
       </c>
       <c r="H15" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="I15" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="16" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16">
         <v>15</v>
       </c>
@@ -1722,28 +1738,28 @@
         <v>15</v>
       </c>
       <c r="C16" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="D16" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="E16" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="F16" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="G16" t="s">
         <v>8</v>
       </c>
       <c r="H16" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="I16" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="17" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="17" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17">
         <v>16</v>
       </c>
@@ -1751,28 +1767,28 @@
         <v>15</v>
       </c>
       <c r="C17" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="D17" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="E17" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="F17" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="G17" t="s">
         <v>9</v>
       </c>
       <c r="H17" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="I17" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="18" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="18" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18">
         <v>17</v>
       </c>
@@ -1780,28 +1796,28 @@
         <v>15</v>
       </c>
       <c r="C18" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="D18" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="E18" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="F18" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="G18" t="s">
         <v>8</v>
       </c>
       <c r="H18" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="I18" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="19" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="19" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19">
         <v>18</v>
       </c>
@@ -1809,28 +1825,28 @@
         <v>15</v>
       </c>
       <c r="C19" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="D19" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="E19" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="F19" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="G19" t="s">
         <v>8</v>
       </c>
       <c r="H19" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="I19" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="20" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="20" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20">
         <v>19</v>
       </c>
@@ -1838,28 +1854,28 @@
         <v>20</v>
       </c>
       <c r="C20" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="D20" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="E20" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="F20" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="G20" t="s">
         <v>7</v>
       </c>
       <c r="H20" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="I20" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="21" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="21" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21">
         <v>20</v>
       </c>
@@ -1867,28 +1883,28 @@
         <v>20</v>
       </c>
       <c r="C21" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="D21" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="E21" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="F21" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="G21" t="s">
         <v>7</v>
       </c>
       <c r="H21" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="I21" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="22" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="22" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22">
         <v>21</v>
       </c>
@@ -1896,16 +1912,16 @@
         <v>20</v>
       </c>
       <c r="C22" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="D22" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="E22" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="F22" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="G22" t="s">
         <v>8</v>
@@ -1917,7 +1933,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="23" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23">
         <v>22</v>
       </c>
@@ -1925,28 +1941,28 @@
         <v>17</v>
       </c>
       <c r="C23" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="D23" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="E23" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="F23" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="G23" t="s">
         <v>9</v>
       </c>
       <c r="H23" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="I23" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="24" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="24" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24">
         <v>23</v>
       </c>
@@ -1954,28 +1970,28 @@
         <v>17</v>
       </c>
       <c r="C24" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="D24" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="E24" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="F24" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="G24" t="s">
         <v>9</v>
       </c>
       <c r="H24" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="I24" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="25" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="25" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25">
         <v>24</v>
       </c>
@@ -1983,28 +1999,28 @@
         <v>17</v>
       </c>
       <c r="C25" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="D25" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="E25" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="F25" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="G25" t="s">
         <v>7</v>
       </c>
       <c r="H25" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="I25" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="26" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="26" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26">
         <v>25</v>
       </c>
@@ -2012,28 +2028,28 @@
         <v>17</v>
       </c>
       <c r="C26" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="D26" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="E26" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="F26" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="G26" t="s">
         <v>8</v>
       </c>
       <c r="H26" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="I26" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="27" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="27" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27">
         <v>26</v>
       </c>
@@ -2041,16 +2057,16 @@
         <v>17</v>
       </c>
       <c r="C27" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="D27" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="E27" t="s">
         <v>12</v>
       </c>
       <c r="F27" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="G27" t="s">
         <v>12</v>
@@ -2062,7 +2078,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="28" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28">
         <v>27</v>
       </c>
@@ -2070,28 +2086,31 @@
         <v>14</v>
       </c>
       <c r="C28" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="D28" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="E28" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="F28" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="G28" t="s">
         <v>9</v>
       </c>
       <c r="H28" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="I28" t="s">
-        <v>149</v>
-      </c>
-    </row>
-    <row r="29" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+        <v>150</v>
+      </c>
+      <c r="J28" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="29" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A29">
         <v>28</v>
       </c>
@@ -2099,28 +2118,31 @@
         <v>14</v>
       </c>
       <c r="C29" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="D29" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="E29" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="F29" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="G29" t="s">
         <v>7</v>
       </c>
       <c r="H29" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="I29" t="s">
-        <v>153</v>
-      </c>
-    </row>
-    <row r="30" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+        <v>154</v>
+      </c>
+      <c r="J29" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="30" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A30">
         <v>29</v>
       </c>
@@ -2128,28 +2150,31 @@
         <v>14</v>
       </c>
       <c r="C30" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="D30" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="E30" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="F30" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="G30" t="s">
         <v>7</v>
       </c>
       <c r="H30" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="I30" t="s">
-        <v>153</v>
-      </c>
-    </row>
-    <row r="31" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+        <v>154</v>
+      </c>
+      <c r="J30" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="31" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A31">
         <v>30</v>
       </c>
@@ -2157,28 +2182,31 @@
         <v>14</v>
       </c>
       <c r="C31" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="D31" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="E31" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="F31" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="G31" t="s">
         <v>7</v>
       </c>
       <c r="H31" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="I31" t="s">
-        <v>159</v>
-      </c>
-    </row>
-    <row r="32" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+        <v>160</v>
+      </c>
+      <c r="J31" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="32" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A32">
         <v>31</v>
       </c>
@@ -2186,28 +2214,28 @@
         <v>14</v>
       </c>
       <c r="C32" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="D32" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="E32" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="F32" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="G32" t="s">
         <v>7</v>
       </c>
       <c r="H32" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="I32" t="s">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="33" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="33" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A33">
         <v>32</v>
       </c>
@@ -2215,28 +2243,28 @@
         <v>14</v>
       </c>
       <c r="C33" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="D33" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="E33" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="F33" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="G33" t="s">
         <v>7</v>
       </c>
       <c r="H33" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="I33" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="34" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="34" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A34">
         <v>33</v>
       </c>
@@ -2244,28 +2272,28 @@
         <v>14</v>
       </c>
       <c r="C34" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="D34" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="E34" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="F34" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="G34" t="s">
         <v>7</v>
       </c>
       <c r="H34" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="I34" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="35" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A35">
         <v>34</v>
       </c>
@@ -2273,28 +2301,28 @@
         <v>24</v>
       </c>
       <c r="C35" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="D35" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="E35" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="F35" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="G35" t="s">
         <v>7</v>
       </c>
       <c r="H35" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="I35" t="s">
-        <v>172</v>
-      </c>
-    </row>
-    <row r="36" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="36" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A36">
         <v>35</v>
       </c>
@@ -2302,28 +2330,28 @@
         <v>24</v>
       </c>
       <c r="C36" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="D36" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="E36" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="F36" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="G36" t="s">
         <v>8</v>
       </c>
       <c r="H36" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="I36" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="37" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="37" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A37">
         <v>36</v>
       </c>
@@ -2331,28 +2359,28 @@
         <v>21</v>
       </c>
       <c r="C37" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="D37" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="E37" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="F37" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="G37" t="s">
         <v>8</v>
       </c>
       <c r="H37" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="I37" t="s">
-        <v>181</v>
-      </c>
-    </row>
-    <row r="38" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="38" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A38">
         <v>37</v>
       </c>
@@ -2360,28 +2388,28 @@
         <v>21</v>
       </c>
       <c r="C38" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="D38" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="E38" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="F38" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="G38" t="s">
         <v>7</v>
       </c>
       <c r="H38" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="I38" t="s">
-        <v>185</v>
-      </c>
-    </row>
-    <row r="39" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="39" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A39">
         <v>38</v>
       </c>
@@ -2389,28 +2417,28 @@
         <v>21</v>
       </c>
       <c r="C39" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="D39" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="E39" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="F39" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="G39" t="s">
         <v>8</v>
       </c>
       <c r="H39" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="I39" t="s">
-        <v>189</v>
-      </c>
-    </row>
-    <row r="40" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="40" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A40">
         <v>39</v>
       </c>
@@ -2418,28 +2446,28 @@
         <v>25</v>
       </c>
       <c r="C40" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="D40" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="E40" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="F40" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="G40" t="s">
         <v>7</v>
       </c>
       <c r="H40" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="I40" t="s">
-        <v>193</v>
-      </c>
-    </row>
-    <row r="41" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="41" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A41">
         <v>40</v>
       </c>
@@ -2447,28 +2475,28 @@
         <v>25</v>
       </c>
       <c r="C41" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="D41" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="E41" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="F41" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="G41" t="s">
         <v>8</v>
       </c>
       <c r="H41" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="I41" t="s">
-        <v>197</v>
-      </c>
-    </row>
-    <row r="42" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="42" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A42">
         <v>41</v>
       </c>
@@ -2476,28 +2504,31 @@
         <v>22</v>
       </c>
       <c r="C42" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="D42" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="E42" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="F42" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="G42" t="s">
         <v>9</v>
       </c>
       <c r="H42" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="I42" t="s">
-        <v>201</v>
-      </c>
-    </row>
-    <row r="43" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+        <v>202</v>
+      </c>
+      <c r="J42" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="43" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A43">
         <v>42</v>
       </c>
@@ -2505,28 +2536,28 @@
         <v>22</v>
       </c>
       <c r="C43" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="D43" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="E43" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="F43" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="G43" t="s">
         <v>7</v>
       </c>
       <c r="H43" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="I43" t="s">
-        <v>204</v>
-      </c>
-    </row>
-    <row r="44" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="44" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A44">
         <v>43</v>
       </c>
@@ -2534,28 +2565,28 @@
         <v>22</v>
       </c>
       <c r="C44" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="D44" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="E44" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="F44" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="G44" t="s">
         <v>7</v>
       </c>
       <c r="H44" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="I44" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="45" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A45">
         <v>44</v>
       </c>
@@ -2563,28 +2594,28 @@
         <v>23</v>
       </c>
       <c r="C45" t="s">
+        <v>210</v>
+      </c>
+      <c r="D45" t="s">
+        <v>211</v>
+      </c>
+      <c r="E45" t="s">
         <v>209</v>
       </c>
-      <c r="D45" t="s">
-        <v>210</v>
-      </c>
-      <c r="E45" t="s">
-        <v>208</v>
-      </c>
       <c r="F45" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="G45" t="s">
         <v>10</v>
       </c>
       <c r="H45" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="I45" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="46" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A46">
         <v>45</v>
       </c>
@@ -2592,28 +2623,28 @@
         <v>23</v>
       </c>
       <c r="C46" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="D46" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="E46" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="F46" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="G46" t="s">
         <v>10</v>
       </c>
       <c r="H46" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="I46" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="47" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A47">
         <v>46</v>
       </c>
@@ -2621,22 +2652,22 @@
         <v>23</v>
       </c>
       <c r="C47" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="D47" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="E47" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="F47" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="G47" t="s">
         <v>8</v>
       </c>
       <c r="H47" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="I47" t="s">
         <v>10</v>
@@ -2646,7 +2677,7 @@
   <autoFilter ref="A1:I47" xr:uid="{00000000-0009-0000-0000-000001000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:I40 A42:I47 A41:B41 D41:I41" numberStoredAsText="1"/>
+    <ignoredError sqref="A1:J9 A11:J27 A10:H10 J10 A32:J41 A28:I28 A29:I31 A43:J47 A42:I42" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: enhance NodalOfficerDashboard and UploaderDashboard with new features and UI improvements
- Added new fields to NodalOfficerDashboard for document details including short title, uploader info, and type-specific fields.
- Improved document relationships handling in NodalOfficerDashboard.
- Updated UploaderDashboard to change active page handling from 'myuploads' to 'dashboard'.
- Introduced a welcome header and quick actions section in UploaderDashboard for better user experience.
- Enhanced layout and styling across various components in UploaderDashboard for improved usability and aesthetics.
- Merged steps in the document upload process for a more streamlined user experience.
- Adjusted input fields and descriptions for clarity and consistency.
</commit_message>
<xml_diff>
--- a/GIGW_DBIM_Compliance_Tasks.xlsx
+++ b/GIGW_DBIM_Compliance_Tasks.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\TOR PROJECT\hlks-demo\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{045DDB39-22C4-4F9F-88EA-E3E89B0D112B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{219FE4E2-0157-43A5-85D1-914E3EF858A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Summary" sheetId="1" r:id="rId1"/>
@@ -32,9 +32,6 @@
     <t>Project</t>
   </si>
   <si>
-    <t>Haryana State Legal Knowledge System (hlks-demo)</t>
-  </si>
-  <si>
     <t>Generated</t>
   </si>
   <si>
@@ -687,14 +684,25 @@
   </si>
   <si>
     <t>Reference</t>
+  </si>
+  <si>
+    <t>Haryana State Digital Knowledge System (hlks-demo)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="12"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -728,9 +736,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1071,7 +1080,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B27"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="28.796875" customWidth="1"/>
     <col min="2" max="2" width="50.796875" customWidth="1"/>
@@ -1087,28 +1096,28 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>2</v>
+        <v>220</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
+        <v>2</v>
+      </c>
+      <c r="B3" t="s">
         <v>3</v>
-      </c>
-      <c r="B3" t="s">
-        <v>4</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
+        <v>4</v>
+      </c>
+      <c r="B5" t="s">
         <v>5</v>
-      </c>
-      <c r="B5" t="s">
-        <v>6</v>
       </c>
     </row>
     <row r="6" spans="1:2" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B6">
         <v>20</v>
@@ -1116,7 +1125,7 @@
     </row>
     <row r="7" spans="1:2" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B7">
         <v>14</v>
@@ -1124,7 +1133,7 @@
     </row>
     <row r="8" spans="1:2" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B8">
         <v>8</v>
@@ -1132,7 +1141,7 @@
     </row>
     <row r="9" spans="1:2" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B9">
         <v>2</v>
@@ -1140,7 +1149,7 @@
     </row>
     <row r="10" spans="1:2" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B10">
         <v>1</v>
@@ -1148,7 +1157,7 @@
     </row>
     <row r="11" spans="1:2" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B11">
         <v>1</v>
@@ -1156,15 +1165,15 @@
     </row>
     <row r="13" spans="1:2" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B13" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="14" spans="1:2" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B14">
         <v>7</v>
@@ -1172,7 +1181,7 @@
     </row>
     <row r="15" spans="1:2" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B15">
         <v>6</v>
@@ -1180,7 +1189,7 @@
     </row>
     <row r="16" spans="1:2" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B16">
         <v>5</v>
@@ -1188,7 +1197,7 @@
     </row>
     <row r="17" spans="1:2" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B17">
         <v>5</v>
@@ -1196,7 +1205,7 @@
     </row>
     <row r="18" spans="1:2" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B18">
         <v>4</v>
@@ -1204,7 +1213,7 @@
     </row>
     <row r="19" spans="1:2" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B19">
         <v>3</v>
@@ -1212,7 +1221,7 @@
     </row>
     <row r="20" spans="1:2" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B20">
         <v>3</v>
@@ -1220,7 +1229,7 @@
     </row>
     <row r="21" spans="1:2" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B21">
         <v>3</v>
@@ -1228,7 +1237,7 @@
     </row>
     <row r="22" spans="1:2" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B22">
         <v>3</v>
@@ -1236,7 +1245,7 @@
     </row>
     <row r="23" spans="1:2" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B23">
         <v>3</v>
@@ -1244,7 +1253,7 @@
     </row>
     <row r="24" spans="1:2" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B24">
         <v>2</v>
@@ -1252,7 +1261,7 @@
     </row>
     <row r="25" spans="1:2" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B25">
         <v>2</v>
@@ -1260,7 +1269,7 @@
     </row>
     <row r="27" spans="1:2" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B27">
         <v>46</v>
@@ -1269,7 +1278,7 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:B27" numberStoredAsText="1"/>
+    <ignoredError sqref="A1:B1 A3:B27 A2" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1277,7 +1286,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:J47"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="6.796875" customWidth="1"/>
     <col min="2" max="2" width="16.796875" customWidth="1"/>
@@ -1290,35 +1299,35 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
+      <c r="A1" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="B1" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="G1" t="s">
+      <c r="H1" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="H1" t="s">
+      <c r="I1" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="I1" t="s">
+      <c r="J1" s="2" t="s">
         <v>35</v>
-      </c>
-      <c r="J1" t="s">
-        <v>36</v>
       </c>
     </row>
     <row r="2" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
@@ -1326,28 +1335,28 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C2" t="s">
+        <v>36</v>
+      </c>
+      <c r="D2" t="s">
         <v>37</v>
       </c>
-      <c r="D2" t="s">
+      <c r="E2" t="s">
         <v>38</v>
       </c>
-      <c r="E2" t="s">
+      <c r="F2" t="s">
         <v>39</v>
       </c>
-      <c r="F2" t="s">
+      <c r="G2" t="s">
+        <v>6</v>
+      </c>
+      <c r="H2" t="s">
         <v>40</v>
       </c>
-      <c r="G2" t="s">
-        <v>7</v>
-      </c>
-      <c r="H2" t="s">
+      <c r="I2" t="s">
         <v>41</v>
-      </c>
-      <c r="I2" t="s">
-        <v>42</v>
       </c>
     </row>
     <row r="3" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
@@ -1355,28 +1364,28 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C3" t="s">
+        <v>42</v>
+      </c>
+      <c r="D3" t="s">
         <v>43</v>
       </c>
-      <c r="D3" t="s">
+      <c r="E3" t="s">
         <v>44</v>
       </c>
-      <c r="E3" t="s">
+      <c r="F3" t="s">
         <v>45</v>
       </c>
-      <c r="F3" t="s">
-        <v>46</v>
-      </c>
       <c r="G3" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="H3" t="s">
+        <v>40</v>
+      </c>
+      <c r="I3" t="s">
         <v>41</v>
-      </c>
-      <c r="I3" t="s">
-        <v>42</v>
       </c>
     </row>
     <row r="4" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
@@ -1384,28 +1393,28 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C4" t="s">
+        <v>46</v>
+      </c>
+      <c r="D4" t="s">
         <v>47</v>
       </c>
-      <c r="D4" t="s">
+      <c r="E4" t="s">
         <v>48</v>
       </c>
-      <c r="E4" t="s">
+      <c r="F4" t="s">
         <v>49</v>
       </c>
-      <c r="F4" t="s">
+      <c r="G4" t="s">
+        <v>6</v>
+      </c>
+      <c r="H4" t="s">
+        <v>40</v>
+      </c>
+      <c r="I4" t="s">
         <v>50</v>
-      </c>
-      <c r="G4" t="s">
-        <v>7</v>
-      </c>
-      <c r="H4" t="s">
-        <v>41</v>
-      </c>
-      <c r="I4" t="s">
-        <v>51</v>
       </c>
     </row>
     <row r="5" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
@@ -1413,31 +1422,31 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C5" t="s">
+        <v>51</v>
+      </c>
+      <c r="D5" t="s">
         <v>52</v>
       </c>
-      <c r="D5" t="s">
+      <c r="E5" t="s">
+        <v>10</v>
+      </c>
+      <c r="F5" t="s">
         <v>53</v>
       </c>
-      <c r="E5" t="s">
-        <v>11</v>
-      </c>
-      <c r="F5" t="s">
+      <c r="G5" t="s">
+        <v>10</v>
+      </c>
+      <c r="H5" t="s">
+        <v>9</v>
+      </c>
+      <c r="I5" t="s">
         <v>54</v>
       </c>
-      <c r="G5" t="s">
-        <v>11</v>
-      </c>
-      <c r="H5" t="s">
+      <c r="J5" s="1" t="s">
         <v>10</v>
-      </c>
-      <c r="I5" t="s">
-        <v>55</v>
-      </c>
-      <c r="J5" s="1" t="s">
-        <v>11</v>
       </c>
     </row>
     <row r="6" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
@@ -1445,28 +1454,28 @@
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C6" t="s">
+        <v>55</v>
+      </c>
+      <c r="D6" t="s">
         <v>56</v>
       </c>
-      <c r="D6" t="s">
+      <c r="E6" t="s">
+        <v>44</v>
+      </c>
+      <c r="F6" t="s">
         <v>57</v>
       </c>
-      <c r="E6" t="s">
-        <v>45</v>
-      </c>
-      <c r="F6" t="s">
+      <c r="G6" t="s">
+        <v>6</v>
+      </c>
+      <c r="H6" t="s">
+        <v>40</v>
+      </c>
+      <c r="I6" t="s">
         <v>58</v>
-      </c>
-      <c r="G6" t="s">
-        <v>7</v>
-      </c>
-      <c r="H6" t="s">
-        <v>41</v>
-      </c>
-      <c r="I6" t="s">
-        <v>59</v>
       </c>
     </row>
     <row r="7" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
@@ -1474,28 +1483,28 @@
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C7" t="s">
+        <v>59</v>
+      </c>
+      <c r="D7" t="s">
         <v>60</v>
       </c>
-      <c r="D7" t="s">
+      <c r="E7" t="s">
+        <v>48</v>
+      </c>
+      <c r="F7" t="s">
         <v>61</v>
       </c>
-      <c r="E7" t="s">
-        <v>49</v>
-      </c>
-      <c r="F7" t="s">
+      <c r="G7" t="s">
+        <v>7</v>
+      </c>
+      <c r="H7" t="s">
         <v>62</v>
       </c>
-      <c r="G7" t="s">
-        <v>8</v>
-      </c>
-      <c r="H7" t="s">
+      <c r="I7" t="s">
         <v>63</v>
-      </c>
-      <c r="I7" t="s">
-        <v>64</v>
       </c>
     </row>
     <row r="8" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
@@ -1503,28 +1512,28 @@
         <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C8" t="s">
+        <v>64</v>
+      </c>
+      <c r="D8" t="s">
         <v>65</v>
       </c>
-      <c r="D8" t="s">
+      <c r="E8" t="s">
+        <v>44</v>
+      </c>
+      <c r="F8" t="s">
         <v>66</v>
       </c>
-      <c r="E8" t="s">
-        <v>45</v>
-      </c>
-      <c r="F8" t="s">
+      <c r="G8" t="s">
+        <v>7</v>
+      </c>
+      <c r="H8" t="s">
         <v>67</v>
       </c>
-      <c r="G8" t="s">
-        <v>8</v>
-      </c>
-      <c r="H8" t="s">
+      <c r="I8" t="s">
         <v>68</v>
-      </c>
-      <c r="I8" t="s">
-        <v>69</v>
       </c>
     </row>
     <row r="9" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
@@ -1532,28 +1541,28 @@
         <v>8</v>
       </c>
       <c r="B9" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C9" t="s">
+        <v>69</v>
+      </c>
+      <c r="D9" t="s">
         <v>70</v>
       </c>
-      <c r="D9" t="s">
+      <c r="E9" t="s">
+        <v>44</v>
+      </c>
+      <c r="F9" t="s">
         <v>71</v>
       </c>
-      <c r="E9" t="s">
-        <v>45</v>
-      </c>
-      <c r="F9" t="s">
+      <c r="G9" t="s">
+        <v>6</v>
+      </c>
+      <c r="H9" t="s">
+        <v>67</v>
+      </c>
+      <c r="I9" t="s">
         <v>72</v>
-      </c>
-      <c r="G9" t="s">
-        <v>7</v>
-      </c>
-      <c r="H9" t="s">
-        <v>68</v>
-      </c>
-      <c r="I9" t="s">
-        <v>73</v>
       </c>
     </row>
     <row r="10" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
@@ -1561,28 +1570,28 @@
         <v>9</v>
       </c>
       <c r="B10" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C10" t="s">
+        <v>73</v>
+      </c>
+      <c r="D10" t="s">
         <v>74</v>
       </c>
-      <c r="D10" t="s">
+      <c r="E10" t="s">
         <v>75</v>
       </c>
-      <c r="E10" t="s">
+      <c r="F10" t="s">
         <v>76</v>
       </c>
-      <c r="F10" t="s">
+      <c r="G10" t="s">
+        <v>8</v>
+      </c>
+      <c r="H10" t="s">
+        <v>67</v>
+      </c>
+      <c r="I10" t="s">
         <v>77</v>
-      </c>
-      <c r="G10" t="s">
-        <v>9</v>
-      </c>
-      <c r="H10" t="s">
-        <v>68</v>
-      </c>
-      <c r="I10" t="s">
-        <v>78</v>
       </c>
     </row>
     <row r="11" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
@@ -1590,28 +1599,28 @@
         <v>10</v>
       </c>
       <c r="B11" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C11" t="s">
+        <v>78</v>
+      </c>
+      <c r="D11" t="s">
         <v>79</v>
       </c>
-      <c r="D11" t="s">
+      <c r="E11" t="s">
+        <v>75</v>
+      </c>
+      <c r="F11" t="s">
         <v>80</v>
       </c>
-      <c r="E11" t="s">
-        <v>76</v>
-      </c>
-      <c r="F11" t="s">
+      <c r="G11" t="s">
+        <v>6</v>
+      </c>
+      <c r="H11" t="s">
+        <v>40</v>
+      </c>
+      <c r="I11" t="s">
         <v>81</v>
-      </c>
-      <c r="G11" t="s">
-        <v>7</v>
-      </c>
-      <c r="H11" t="s">
-        <v>41</v>
-      </c>
-      <c r="I11" t="s">
-        <v>82</v>
       </c>
     </row>
     <row r="12" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
@@ -1619,28 +1628,28 @@
         <v>11</v>
       </c>
       <c r="B12" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C12" t="s">
+        <v>82</v>
+      </c>
+      <c r="D12" t="s">
         <v>83</v>
       </c>
-      <c r="D12" t="s">
+      <c r="E12" t="s">
+        <v>44</v>
+      </c>
+      <c r="F12" t="s">
         <v>84</v>
       </c>
-      <c r="E12" t="s">
-        <v>45</v>
-      </c>
-      <c r="F12" t="s">
+      <c r="G12" t="s">
+        <v>8</v>
+      </c>
+      <c r="H12" t="s">
+        <v>67</v>
+      </c>
+      <c r="I12" t="s">
         <v>85</v>
-      </c>
-      <c r="G12" t="s">
-        <v>9</v>
-      </c>
-      <c r="H12" t="s">
-        <v>68</v>
-      </c>
-      <c r="I12" t="s">
-        <v>86</v>
       </c>
     </row>
     <row r="13" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
@@ -1648,28 +1657,28 @@
         <v>12</v>
       </c>
       <c r="B13" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C13" t="s">
+        <v>86</v>
+      </c>
+      <c r="D13" t="s">
         <v>87</v>
       </c>
-      <c r="D13" t="s">
+      <c r="E13" t="s">
         <v>88</v>
       </c>
-      <c r="E13" t="s">
+      <c r="F13" t="s">
         <v>89</v>
       </c>
-      <c r="F13" t="s">
+      <c r="G13" t="s">
+        <v>6</v>
+      </c>
+      <c r="H13" t="s">
+        <v>40</v>
+      </c>
+      <c r="I13" t="s">
         <v>90</v>
-      </c>
-      <c r="G13" t="s">
-        <v>7</v>
-      </c>
-      <c r="H13" t="s">
-        <v>41</v>
-      </c>
-      <c r="I13" t="s">
-        <v>91</v>
       </c>
     </row>
     <row r="14" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
@@ -1677,28 +1686,28 @@
         <v>13</v>
       </c>
       <c r="B14" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C14" t="s">
+        <v>91</v>
+      </c>
+      <c r="D14" t="s">
         <v>92</v>
       </c>
-      <c r="D14" t="s">
+      <c r="E14" t="s">
         <v>93</v>
       </c>
-      <c r="E14" t="s">
+      <c r="F14" t="s">
         <v>94</v>
       </c>
-      <c r="F14" t="s">
+      <c r="G14" t="s">
+        <v>7</v>
+      </c>
+      <c r="H14" t="s">
+        <v>40</v>
+      </c>
+      <c r="I14" t="s">
         <v>95</v>
-      </c>
-      <c r="G14" t="s">
-        <v>8</v>
-      </c>
-      <c r="H14" t="s">
-        <v>41</v>
-      </c>
-      <c r="I14" t="s">
-        <v>96</v>
       </c>
     </row>
     <row r="15" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
@@ -1706,28 +1715,28 @@
         <v>14</v>
       </c>
       <c r="B15" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C15" t="s">
+        <v>96</v>
+      </c>
+      <c r="D15" t="s">
         <v>97</v>
       </c>
-      <c r="D15" t="s">
+      <c r="E15" t="s">
+        <v>75</v>
+      </c>
+      <c r="F15" t="s">
         <v>98</v>
       </c>
-      <c r="E15" t="s">
-        <v>76</v>
-      </c>
-      <c r="F15" t="s">
+      <c r="G15" t="s">
+        <v>8</v>
+      </c>
+      <c r="H15" t="s">
+        <v>62</v>
+      </c>
+      <c r="I15" t="s">
         <v>99</v>
-      </c>
-      <c r="G15" t="s">
-        <v>9</v>
-      </c>
-      <c r="H15" t="s">
-        <v>63</v>
-      </c>
-      <c r="I15" t="s">
-        <v>100</v>
       </c>
     </row>
     <row r="16" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
@@ -1735,28 +1744,28 @@
         <v>15</v>
       </c>
       <c r="B16" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C16" t="s">
+        <v>100</v>
+      </c>
+      <c r="D16" t="s">
+        <v>92</v>
+      </c>
+      <c r="E16" t="s">
+        <v>44</v>
+      </c>
+      <c r="F16" t="s">
         <v>101</v>
       </c>
-      <c r="D16" t="s">
-        <v>93</v>
-      </c>
-      <c r="E16" t="s">
-        <v>45</v>
-      </c>
-      <c r="F16" t="s">
-        <v>102</v>
-      </c>
       <c r="G16" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="H16" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="I16" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="17" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
@@ -1764,28 +1773,28 @@
         <v>16</v>
       </c>
       <c r="B17" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C17" t="s">
+        <v>102</v>
+      </c>
+      <c r="D17" t="s">
         <v>103</v>
       </c>
-      <c r="D17" t="s">
+      <c r="E17" t="s">
+        <v>75</v>
+      </c>
+      <c r="F17" t="s">
         <v>104</v>
       </c>
-      <c r="E17" t="s">
-        <v>76</v>
-      </c>
-      <c r="F17" t="s">
+      <c r="G17" t="s">
+        <v>8</v>
+      </c>
+      <c r="H17" t="s">
+        <v>40</v>
+      </c>
+      <c r="I17" t="s">
         <v>105</v>
-      </c>
-      <c r="G17" t="s">
-        <v>9</v>
-      </c>
-      <c r="H17" t="s">
-        <v>41</v>
-      </c>
-      <c r="I17" t="s">
-        <v>106</v>
       </c>
     </row>
     <row r="18" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
@@ -1793,28 +1802,28 @@
         <v>17</v>
       </c>
       <c r="B18" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C18" t="s">
+        <v>106</v>
+      </c>
+      <c r="D18" t="s">
         <v>107</v>
       </c>
-      <c r="D18" t="s">
+      <c r="E18" t="s">
+        <v>75</v>
+      </c>
+      <c r="F18" t="s">
         <v>108</v>
       </c>
-      <c r="E18" t="s">
-        <v>76</v>
-      </c>
-      <c r="F18" t="s">
+      <c r="G18" t="s">
+        <v>7</v>
+      </c>
+      <c r="H18" t="s">
+        <v>67</v>
+      </c>
+      <c r="I18" t="s">
         <v>109</v>
-      </c>
-      <c r="G18" t="s">
-        <v>8</v>
-      </c>
-      <c r="H18" t="s">
-        <v>68</v>
-      </c>
-      <c r="I18" t="s">
-        <v>110</v>
       </c>
     </row>
     <row r="19" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
@@ -1822,28 +1831,28 @@
         <v>18</v>
       </c>
       <c r="B19" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C19" t="s">
+        <v>110</v>
+      </c>
+      <c r="D19" t="s">
+        <v>92</v>
+      </c>
+      <c r="E19" t="s">
+        <v>44</v>
+      </c>
+      <c r="F19" t="s">
         <v>111</v>
       </c>
-      <c r="D19" t="s">
-        <v>93</v>
-      </c>
-      <c r="E19" t="s">
-        <v>45</v>
-      </c>
-      <c r="F19" t="s">
+      <c r="G19" t="s">
+        <v>7</v>
+      </c>
+      <c r="H19" t="s">
+        <v>67</v>
+      </c>
+      <c r="I19" t="s">
         <v>112</v>
-      </c>
-      <c r="G19" t="s">
-        <v>8</v>
-      </c>
-      <c r="H19" t="s">
-        <v>68</v>
-      </c>
-      <c r="I19" t="s">
-        <v>113</v>
       </c>
     </row>
     <row r="20" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
@@ -1851,28 +1860,28 @@
         <v>19</v>
       </c>
       <c r="B20" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C20" t="s">
+        <v>113</v>
+      </c>
+      <c r="D20" t="s">
         <v>114</v>
       </c>
-      <c r="D20" t="s">
+      <c r="E20" t="s">
         <v>115</v>
       </c>
-      <c r="E20" t="s">
+      <c r="F20" t="s">
         <v>116</v>
       </c>
-      <c r="F20" t="s">
+      <c r="G20" t="s">
+        <v>6</v>
+      </c>
+      <c r="H20" t="s">
+        <v>67</v>
+      </c>
+      <c r="I20" t="s">
         <v>117</v>
-      </c>
-      <c r="G20" t="s">
-        <v>7</v>
-      </c>
-      <c r="H20" t="s">
-        <v>68</v>
-      </c>
-      <c r="I20" t="s">
-        <v>118</v>
       </c>
     </row>
     <row r="21" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
@@ -1880,28 +1889,28 @@
         <v>20</v>
       </c>
       <c r="B21" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C21" t="s">
+        <v>118</v>
+      </c>
+      <c r="D21" t="s">
         <v>119</v>
       </c>
-      <c r="D21" t="s">
+      <c r="E21" t="s">
+        <v>44</v>
+      </c>
+      <c r="F21" t="s">
         <v>120</v>
       </c>
-      <c r="E21" t="s">
-        <v>45</v>
-      </c>
-      <c r="F21" t="s">
+      <c r="G21" t="s">
+        <v>6</v>
+      </c>
+      <c r="H21" t="s">
+        <v>40</v>
+      </c>
+      <c r="I21" t="s">
         <v>121</v>
-      </c>
-      <c r="G21" t="s">
-        <v>7</v>
-      </c>
-      <c r="H21" t="s">
-        <v>41</v>
-      </c>
-      <c r="I21" t="s">
-        <v>122</v>
       </c>
     </row>
     <row r="22" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
@@ -1909,28 +1918,28 @@
         <v>21</v>
       </c>
       <c r="B22" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C22" t="s">
+        <v>122</v>
+      </c>
+      <c r="D22" t="s">
         <v>123</v>
       </c>
-      <c r="D22" t="s">
+      <c r="E22" t="s">
         <v>124</v>
       </c>
-      <c r="E22" t="s">
+      <c r="F22" t="s">
         <v>125</v>
       </c>
-      <c r="F22" t="s">
-        <v>126</v>
-      </c>
       <c r="G22" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="H22" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="I22" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="23" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
@@ -1938,28 +1947,28 @@
         <v>22</v>
       </c>
       <c r="B23" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C23" t="s">
+        <v>126</v>
+      </c>
+      <c r="D23" t="s">
         <v>127</v>
       </c>
-      <c r="D23" t="s">
+      <c r="E23" t="s">
+        <v>75</v>
+      </c>
+      <c r="F23" t="s">
         <v>128</v>
       </c>
-      <c r="E23" t="s">
-        <v>76</v>
-      </c>
-      <c r="F23" t="s">
+      <c r="G23" t="s">
+        <v>8</v>
+      </c>
+      <c r="H23" t="s">
+        <v>62</v>
+      </c>
+      <c r="I23" t="s">
         <v>129</v>
-      </c>
-      <c r="G23" t="s">
-        <v>9</v>
-      </c>
-      <c r="H23" t="s">
-        <v>63</v>
-      </c>
-      <c r="I23" t="s">
-        <v>130</v>
       </c>
     </row>
     <row r="24" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
@@ -1967,28 +1976,28 @@
         <v>23</v>
       </c>
       <c r="B24" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C24" t="s">
+        <v>130</v>
+      </c>
+      <c r="D24" t="s">
         <v>131</v>
       </c>
-      <c r="D24" t="s">
+      <c r="E24" t="s">
+        <v>75</v>
+      </c>
+      <c r="F24" t="s">
         <v>132</v>
       </c>
-      <c r="E24" t="s">
-        <v>76</v>
-      </c>
-      <c r="F24" t="s">
+      <c r="G24" t="s">
+        <v>8</v>
+      </c>
+      <c r="H24" t="s">
+        <v>67</v>
+      </c>
+      <c r="I24" t="s">
         <v>133</v>
-      </c>
-      <c r="G24" t="s">
-        <v>9</v>
-      </c>
-      <c r="H24" t="s">
-        <v>68</v>
-      </c>
-      <c r="I24" t="s">
-        <v>134</v>
       </c>
     </row>
     <row r="25" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
@@ -1996,28 +2005,28 @@
         <v>24</v>
       </c>
       <c r="B25" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C25" t="s">
+        <v>134</v>
+      </c>
+      <c r="D25" t="s">
         <v>135</v>
       </c>
-      <c r="D25" t="s">
+      <c r="E25" t="s">
+        <v>48</v>
+      </c>
+      <c r="F25" t="s">
         <v>136</v>
       </c>
-      <c r="E25" t="s">
-        <v>49</v>
-      </c>
-      <c r="F25" t="s">
+      <c r="G25" t="s">
+        <v>6</v>
+      </c>
+      <c r="H25" t="s">
+        <v>67</v>
+      </c>
+      <c r="I25" t="s">
         <v>137</v>
-      </c>
-      <c r="G25" t="s">
-        <v>7</v>
-      </c>
-      <c r="H25" t="s">
-        <v>68</v>
-      </c>
-      <c r="I25" t="s">
-        <v>138</v>
       </c>
     </row>
     <row r="26" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
@@ -2025,28 +2034,28 @@
         <v>25</v>
       </c>
       <c r="B26" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C26" t="s">
+        <v>138</v>
+      </c>
+      <c r="D26" t="s">
         <v>139</v>
       </c>
-      <c r="D26" t="s">
+      <c r="E26" t="s">
         <v>140</v>
       </c>
-      <c r="E26" t="s">
+      <c r="F26" t="s">
         <v>141</v>
       </c>
-      <c r="F26" t="s">
+      <c r="G26" t="s">
+        <v>7</v>
+      </c>
+      <c r="H26" t="s">
+        <v>67</v>
+      </c>
+      <c r="I26" t="s">
         <v>142</v>
-      </c>
-      <c r="G26" t="s">
-        <v>8</v>
-      </c>
-      <c r="H26" t="s">
-        <v>68</v>
-      </c>
-      <c r="I26" t="s">
-        <v>143</v>
       </c>
     </row>
     <row r="27" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
@@ -2054,28 +2063,28 @@
         <v>26</v>
       </c>
       <c r="B27" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C27" t="s">
+        <v>143</v>
+      </c>
+      <c r="D27" t="s">
         <v>144</v>
       </c>
-      <c r="D27" t="s">
+      <c r="E27" t="s">
+        <v>11</v>
+      </c>
+      <c r="F27" t="s">
         <v>145</v>
       </c>
-      <c r="E27" t="s">
-        <v>12</v>
-      </c>
-      <c r="F27" t="s">
-        <v>146</v>
-      </c>
       <c r="G27" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="H27" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="I27" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="28" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
@@ -2083,31 +2092,31 @@
         <v>27</v>
       </c>
       <c r="B28" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C28" t="s">
+        <v>146</v>
+      </c>
+      <c r="D28" t="s">
         <v>147</v>
       </c>
-      <c r="D28" t="s">
+      <c r="E28" t="s">
+        <v>44</v>
+      </c>
+      <c r="F28" t="s">
         <v>148</v>
       </c>
-      <c r="E28" t="s">
-        <v>45</v>
-      </c>
-      <c r="F28" t="s">
+      <c r="G28" t="s">
+        <v>8</v>
+      </c>
+      <c r="H28" t="s">
+        <v>40</v>
+      </c>
+      <c r="I28" t="s">
         <v>149</v>
       </c>
-      <c r="G28" t="s">
-        <v>9</v>
-      </c>
-      <c r="H28" t="s">
-        <v>41</v>
-      </c>
-      <c r="I28" t="s">
-        <v>150</v>
-      </c>
       <c r="J28" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="29" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
@@ -2115,31 +2124,31 @@
         <v>28</v>
       </c>
       <c r="B29" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C29" t="s">
+        <v>150</v>
+      </c>
+      <c r="D29" t="s">
         <v>151</v>
       </c>
-      <c r="D29" t="s">
+      <c r="E29" t="s">
+        <v>44</v>
+      </c>
+      <c r="F29" t="s">
         <v>152</v>
       </c>
-      <c r="E29" t="s">
-        <v>45</v>
-      </c>
-      <c r="F29" t="s">
+      <c r="G29" t="s">
+        <v>6</v>
+      </c>
+      <c r="H29" t="s">
+        <v>67</v>
+      </c>
+      <c r="I29" t="s">
         <v>153</v>
       </c>
-      <c r="G29" t="s">
-        <v>7</v>
-      </c>
-      <c r="H29" t="s">
-        <v>68</v>
-      </c>
-      <c r="I29" t="s">
-        <v>154</v>
-      </c>
       <c r="J29" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="30" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
@@ -2147,31 +2156,31 @@
         <v>29</v>
       </c>
       <c r="B30" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C30" t="s">
+        <v>154</v>
+      </c>
+      <c r="D30" t="s">
+        <v>151</v>
+      </c>
+      <c r="E30" t="s">
+        <v>44</v>
+      </c>
+      <c r="F30" t="s">
         <v>155</v>
       </c>
-      <c r="D30" t="s">
-        <v>152</v>
-      </c>
-      <c r="E30" t="s">
-        <v>45</v>
-      </c>
-      <c r="F30" t="s">
-        <v>156</v>
-      </c>
       <c r="G30" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H30" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="I30" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="J30" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="31" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
@@ -2179,31 +2188,31 @@
         <v>30</v>
       </c>
       <c r="B31" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C31" t="s">
+        <v>156</v>
+      </c>
+      <c r="D31" t="s">
         <v>157</v>
       </c>
-      <c r="D31" t="s">
+      <c r="E31" t="s">
+        <v>75</v>
+      </c>
+      <c r="F31" t="s">
         <v>158</v>
       </c>
-      <c r="E31" t="s">
-        <v>76</v>
-      </c>
-      <c r="F31" t="s">
+      <c r="G31" t="s">
+        <v>6</v>
+      </c>
+      <c r="H31" t="s">
+        <v>40</v>
+      </c>
+      <c r="I31" t="s">
         <v>159</v>
       </c>
-      <c r="G31" t="s">
-        <v>7</v>
-      </c>
-      <c r="H31" t="s">
-        <v>41</v>
-      </c>
-      <c r="I31" t="s">
-        <v>160</v>
-      </c>
       <c r="J31" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="32" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
@@ -2211,28 +2220,28 @@
         <v>31</v>
       </c>
       <c r="B32" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C32" t="s">
+        <v>160</v>
+      </c>
+      <c r="D32" t="s">
         <v>161</v>
       </c>
-      <c r="D32" t="s">
+      <c r="E32" t="s">
+        <v>44</v>
+      </c>
+      <c r="F32" t="s">
         <v>162</v>
       </c>
-      <c r="E32" t="s">
-        <v>45</v>
-      </c>
-      <c r="F32" t="s">
+      <c r="G32" t="s">
+        <v>6</v>
+      </c>
+      <c r="H32" t="s">
+        <v>67</v>
+      </c>
+      <c r="I32" t="s">
         <v>163</v>
-      </c>
-      <c r="G32" t="s">
-        <v>7</v>
-      </c>
-      <c r="H32" t="s">
-        <v>68</v>
-      </c>
-      <c r="I32" t="s">
-        <v>164</v>
       </c>
     </row>
     <row r="33" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
@@ -2240,28 +2249,28 @@
         <v>32</v>
       </c>
       <c r="B33" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C33" t="s">
+        <v>164</v>
+      </c>
+      <c r="D33" t="s">
+        <v>147</v>
+      </c>
+      <c r="E33" t="s">
+        <v>44</v>
+      </c>
+      <c r="F33" t="s">
         <v>165</v>
       </c>
-      <c r="D33" t="s">
-        <v>148</v>
-      </c>
-      <c r="E33" t="s">
-        <v>45</v>
-      </c>
-      <c r="F33" t="s">
-        <v>166</v>
-      </c>
       <c r="G33" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H33" t="s">
+        <v>40</v>
+      </c>
+      <c r="I33" t="s">
         <v>41</v>
-      </c>
-      <c r="I33" t="s">
-        <v>42</v>
       </c>
     </row>
     <row r="34" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
@@ -2269,28 +2278,28 @@
         <v>33</v>
       </c>
       <c r="B34" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C34" t="s">
+        <v>166</v>
+      </c>
+      <c r="D34" t="s">
         <v>167</v>
       </c>
-      <c r="D34" t="s">
+      <c r="E34" t="s">
+        <v>48</v>
+      </c>
+      <c r="F34" t="s">
         <v>168</v>
       </c>
-      <c r="E34" t="s">
-        <v>49</v>
-      </c>
-      <c r="F34" t="s">
-        <v>169</v>
-      </c>
       <c r="G34" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H34" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="I34" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="35" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
@@ -2298,28 +2307,28 @@
         <v>34</v>
       </c>
       <c r="B35" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C35" t="s">
+        <v>169</v>
+      </c>
+      <c r="D35" t="s">
         <v>170</v>
       </c>
-      <c r="D35" t="s">
+      <c r="E35" t="s">
+        <v>44</v>
+      </c>
+      <c r="F35" t="s">
         <v>171</v>
       </c>
-      <c r="E35" t="s">
-        <v>45</v>
-      </c>
-      <c r="F35" t="s">
+      <c r="G35" t="s">
+        <v>6</v>
+      </c>
+      <c r="H35" t="s">
+        <v>62</v>
+      </c>
+      <c r="I35" t="s">
         <v>172</v>
-      </c>
-      <c r="G35" t="s">
-        <v>7</v>
-      </c>
-      <c r="H35" t="s">
-        <v>63</v>
-      </c>
-      <c r="I35" t="s">
-        <v>173</v>
       </c>
     </row>
     <row r="36" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
@@ -2327,28 +2336,28 @@
         <v>35</v>
       </c>
       <c r="B36" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C36" t="s">
+        <v>173</v>
+      </c>
+      <c r="D36" t="s">
         <v>174</v>
       </c>
-      <c r="D36" t="s">
+      <c r="E36" t="s">
         <v>175</v>
       </c>
-      <c r="E36" t="s">
+      <c r="F36" t="s">
         <v>176</v>
       </c>
-      <c r="F36" t="s">
+      <c r="G36" t="s">
+        <v>7</v>
+      </c>
+      <c r="H36" t="s">
+        <v>40</v>
+      </c>
+      <c r="I36" t="s">
         <v>177</v>
-      </c>
-      <c r="G36" t="s">
-        <v>8</v>
-      </c>
-      <c r="H36" t="s">
-        <v>41</v>
-      </c>
-      <c r="I36" t="s">
-        <v>178</v>
       </c>
     </row>
     <row r="37" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
@@ -2356,28 +2365,28 @@
         <v>36</v>
       </c>
       <c r="B37" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C37" t="s">
+        <v>178</v>
+      </c>
+      <c r="D37" t="s">
         <v>179</v>
       </c>
-      <c r="D37" t="s">
+      <c r="E37" t="s">
+        <v>48</v>
+      </c>
+      <c r="F37" t="s">
         <v>180</v>
       </c>
-      <c r="E37" t="s">
-        <v>49</v>
-      </c>
-      <c r="F37" t="s">
+      <c r="G37" t="s">
+        <v>7</v>
+      </c>
+      <c r="H37" t="s">
+        <v>40</v>
+      </c>
+      <c r="I37" t="s">
         <v>181</v>
-      </c>
-      <c r="G37" t="s">
-        <v>8</v>
-      </c>
-      <c r="H37" t="s">
-        <v>41</v>
-      </c>
-      <c r="I37" t="s">
-        <v>182</v>
       </c>
     </row>
     <row r="38" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
@@ -2385,28 +2394,28 @@
         <v>37</v>
       </c>
       <c r="B38" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C38" t="s">
+        <v>182</v>
+      </c>
+      <c r="D38" t="s">
         <v>183</v>
       </c>
-      <c r="D38" t="s">
+      <c r="E38" t="s">
+        <v>115</v>
+      </c>
+      <c r="F38" t="s">
         <v>184</v>
       </c>
-      <c r="E38" t="s">
-        <v>116</v>
-      </c>
-      <c r="F38" t="s">
+      <c r="G38" t="s">
+        <v>6</v>
+      </c>
+      <c r="H38" t="s">
+        <v>67</v>
+      </c>
+      <c r="I38" t="s">
         <v>185</v>
-      </c>
-      <c r="G38" t="s">
-        <v>7</v>
-      </c>
-      <c r="H38" t="s">
-        <v>68</v>
-      </c>
-      <c r="I38" t="s">
-        <v>186</v>
       </c>
     </row>
     <row r="39" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
@@ -2414,28 +2423,28 @@
         <v>38</v>
       </c>
       <c r="B39" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C39" t="s">
+        <v>186</v>
+      </c>
+      <c r="D39" t="s">
         <v>187</v>
       </c>
-      <c r="D39" t="s">
+      <c r="E39" t="s">
+        <v>75</v>
+      </c>
+      <c r="F39" t="s">
         <v>188</v>
       </c>
-      <c r="E39" t="s">
-        <v>76</v>
-      </c>
-      <c r="F39" t="s">
+      <c r="G39" t="s">
+        <v>7</v>
+      </c>
+      <c r="H39" t="s">
+        <v>67</v>
+      </c>
+      <c r="I39" t="s">
         <v>189</v>
-      </c>
-      <c r="G39" t="s">
-        <v>8</v>
-      </c>
-      <c r="H39" t="s">
-        <v>68</v>
-      </c>
-      <c r="I39" t="s">
-        <v>190</v>
       </c>
     </row>
     <row r="40" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
@@ -2443,28 +2452,28 @@
         <v>39</v>
       </c>
       <c r="B40" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C40" t="s">
+        <v>190</v>
+      </c>
+      <c r="D40" t="s">
         <v>191</v>
       </c>
-      <c r="D40" t="s">
+      <c r="E40" t="s">
+        <v>44</v>
+      </c>
+      <c r="F40" t="s">
         <v>192</v>
       </c>
-      <c r="E40" t="s">
-        <v>45</v>
-      </c>
-      <c r="F40" t="s">
+      <c r="G40" t="s">
+        <v>6</v>
+      </c>
+      <c r="H40" t="s">
+        <v>67</v>
+      </c>
+      <c r="I40" t="s">
         <v>193</v>
-      </c>
-      <c r="G40" t="s">
-        <v>7</v>
-      </c>
-      <c r="H40" t="s">
-        <v>68</v>
-      </c>
-      <c r="I40" t="s">
-        <v>194</v>
       </c>
     </row>
     <row r="41" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
@@ -2472,28 +2481,28 @@
         <v>40</v>
       </c>
       <c r="B41" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C41" t="s">
+        <v>194</v>
+      </c>
+      <c r="D41" t="s">
         <v>195</v>
       </c>
-      <c r="D41" t="s">
+      <c r="E41" t="s">
+        <v>44</v>
+      </c>
+      <c r="F41" t="s">
         <v>196</v>
       </c>
-      <c r="E41" t="s">
-        <v>45</v>
-      </c>
-      <c r="F41" t="s">
+      <c r="G41" t="s">
+        <v>7</v>
+      </c>
+      <c r="H41" t="s">
+        <v>67</v>
+      </c>
+      <c r="I41" t="s">
         <v>197</v>
-      </c>
-      <c r="G41" t="s">
-        <v>8</v>
-      </c>
-      <c r="H41" t="s">
-        <v>68</v>
-      </c>
-      <c r="I41" t="s">
-        <v>198</v>
       </c>
     </row>
     <row r="42" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
@@ -2501,31 +2510,31 @@
         <v>41</v>
       </c>
       <c r="B42" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C42" t="s">
+        <v>198</v>
+      </c>
+      <c r="D42" t="s">
         <v>199</v>
       </c>
-      <c r="D42" t="s">
+      <c r="E42" t="s">
+        <v>75</v>
+      </c>
+      <c r="F42" t="s">
         <v>200</v>
       </c>
-      <c r="E42" t="s">
-        <v>76</v>
-      </c>
-      <c r="F42" t="s">
+      <c r="G42" t="s">
+        <v>8</v>
+      </c>
+      <c r="H42" t="s">
+        <v>67</v>
+      </c>
+      <c r="I42" t="s">
         <v>201</v>
       </c>
-      <c r="G42" t="s">
-        <v>9</v>
-      </c>
-      <c r="H42" t="s">
-        <v>68</v>
-      </c>
-      <c r="I42" t="s">
-        <v>202</v>
-      </c>
       <c r="J42" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="43" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
@@ -2533,28 +2542,28 @@
         <v>42</v>
       </c>
       <c r="B43" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C43" t="s">
+        <v>202</v>
+      </c>
+      <c r="D43" t="s">
+        <v>157</v>
+      </c>
+      <c r="E43" t="s">
+        <v>44</v>
+      </c>
+      <c r="F43" t="s">
         <v>203</v>
       </c>
-      <c r="D43" t="s">
-        <v>158</v>
-      </c>
-      <c r="E43" t="s">
-        <v>45</v>
-      </c>
-      <c r="F43" t="s">
+      <c r="G43" t="s">
+        <v>6</v>
+      </c>
+      <c r="H43" t="s">
+        <v>67</v>
+      </c>
+      <c r="I43" t="s">
         <v>204</v>
-      </c>
-      <c r="G43" t="s">
-        <v>7</v>
-      </c>
-      <c r="H43" t="s">
-        <v>68</v>
-      </c>
-      <c r="I43" t="s">
-        <v>205</v>
       </c>
     </row>
     <row r="44" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
@@ -2562,28 +2571,28 @@
         <v>43</v>
       </c>
       <c r="B44" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C44" t="s">
+        <v>205</v>
+      </c>
+      <c r="D44" t="s">
+        <v>157</v>
+      </c>
+      <c r="E44" t="s">
         <v>206</v>
       </c>
-      <c r="D44" t="s">
-        <v>158</v>
-      </c>
-      <c r="E44" t="s">
+      <c r="F44" t="s">
         <v>207</v>
       </c>
-      <c r="F44" t="s">
+      <c r="G44" t="s">
+        <v>6</v>
+      </c>
+      <c r="H44" t="s">
         <v>208</v>
       </c>
-      <c r="G44" t="s">
-        <v>7</v>
-      </c>
-      <c r="H44" t="s">
-        <v>209</v>
-      </c>
       <c r="I44" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="45" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
@@ -2591,28 +2600,28 @@
         <v>44</v>
       </c>
       <c r="B45" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C45" t="s">
+        <v>209</v>
+      </c>
+      <c r="D45" t="s">
         <v>210</v>
       </c>
-      <c r="D45" t="s">
+      <c r="E45" t="s">
+        <v>208</v>
+      </c>
+      <c r="F45" t="s">
         <v>211</v>
       </c>
-      <c r="E45" t="s">
-        <v>209</v>
-      </c>
-      <c r="F45" t="s">
-        <v>212</v>
-      </c>
       <c r="G45" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="H45" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="I45" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="46" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
@@ -2620,28 +2629,28 @@
         <v>45</v>
       </c>
       <c r="B46" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C46" t="s">
+        <v>212</v>
+      </c>
+      <c r="D46" t="s">
         <v>213</v>
       </c>
-      <c r="D46" t="s">
+      <c r="E46" t="s">
+        <v>208</v>
+      </c>
+      <c r="F46" t="s">
         <v>214</v>
       </c>
-      <c r="E46" t="s">
-        <v>209</v>
-      </c>
-      <c r="F46" t="s">
-        <v>215</v>
-      </c>
       <c r="G46" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="H46" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="I46" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="47" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
@@ -2649,35 +2658,35 @@
         <v>46</v>
       </c>
       <c r="B47" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C47" t="s">
+        <v>215</v>
+      </c>
+      <c r="D47" t="s">
         <v>216</v>
       </c>
-      <c r="D47" t="s">
+      <c r="E47" t="s">
         <v>217</v>
       </c>
-      <c r="E47" t="s">
+      <c r="F47" t="s">
         <v>218</v>
       </c>
-      <c r="F47" t="s">
+      <c r="G47" t="s">
+        <v>7</v>
+      </c>
+      <c r="H47" t="s">
         <v>219</v>
       </c>
-      <c r="G47" t="s">
-        <v>8</v>
-      </c>
-      <c r="H47" t="s">
-        <v>220</v>
-      </c>
       <c r="I47" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:I47" xr:uid="{00000000-0009-0000-0000-000001000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:J9 A11:J27 A10:H10 J10 A32:J41 A28:I28 A29:I31 A43:J47 A42:I42" numberStoredAsText="1"/>
+    <ignoredError sqref="A1:J9 A11:J27 A10:H10 J10 A32:J41 A28:I28 A29:I31 A44:J47 A42:I42 A43:B43 D43:J43" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Refactor UploaderDashboard to use centralized type-specific field keys and improve DocViewModal display logic
- Replaced hardcoded type-specific fields in UploaderDashboard with constants from docTypeFields.
- Updated DocViewModal to always show all fields, even if empty, for better visibility.
- Enhanced layout consistency in DocViewModal for both common and type-specific fields.
- Added build date definition in vite.config.js for automatic deployment date tracking.
</commit_message>
<xml_diff>
--- a/GIGW_DBIM_Compliance_Tasks.xlsx
+++ b/GIGW_DBIM_Compliance_Tasks.xlsx
@@ -1623,47 +1623,52 @@
       </c>
     </row>
     <row r="17" ht="15.6" customHeight="1">
-      <c r="A17" t="n">
+      <c r="A17" s="8" t="n">
         <v>16</v>
       </c>
-      <c r="B17" t="inlineStr">
+      <c r="B17" s="8" t="inlineStr">
         <is>
           <t>Footer</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr">
+      <c r="C17" s="8" t="inlineStr">
         <is>
           <t>RTI (Right to Information) link in footer/Connect section</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr">
+      <c r="D17" s="8" t="inlineStr">
         <is>
           <t>GIGW mandatory</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>Missing</t>
-        </is>
-      </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>No RTI link/page exists (RTI only appears as legal-document content in mock data)</t>
-        </is>
-      </c>
-      <c r="G17" t="inlineStr">
+      <c r="E17" s="8" t="inlineStr">
+        <is>
+          <t>Compliant</t>
+        </is>
+      </c>
+      <c r="F17" s="8" t="inlineStr">
+        <is>
+          <t>Footer's "Help &amp; Support" section already includes a "Right to Information" link (Footer.jsx, pageKey 'rti'), which opens a full RTI content page via FooterInfoModal.jsx covering the RTI Act 2005, how to file a request (via the Feedback/Contact route to the relevant department's PIO), and the first-appeal process. Not just mock legal-document content — a real, dedicated RTI page.</t>
+        </is>
+      </c>
+      <c r="G17" s="8" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="H17" t="inlineStr">
+      <c r="H17" s="8" t="inlineStr">
         <is>
           <t>S</t>
         </is>
       </c>
-      <c r="I17" t="inlineStr">
+      <c r="I17" s="8" t="inlineStr">
         <is>
           <t>Footer.jsx + new RTI page</t>
+        </is>
+      </c>
+      <c r="J17" s="8" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -1713,47 +1718,52 @@
       </c>
     </row>
     <row r="19" ht="15.6" customHeight="1">
-      <c r="A19" t="n">
+      <c r="A19" s="8" t="n">
         <v>18</v>
       </c>
-      <c r="B19" t="inlineStr">
+      <c r="B19" s="8" t="inlineStr">
         <is>
           <t>Footer</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr">
+      <c r="C19" s="8" t="inlineStr">
         <is>
           <t>'Last Updated On' date reflecting latest content update</t>
         </is>
       </c>
-      <c r="D19" t="inlineStr">
+      <c r="D19" s="8" t="inlineStr">
         <is>
           <t>DBIM 5.6</t>
         </is>
       </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>Partial</t>
-        </is>
-      </c>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>A single static date is hardcoded site-wide instead of being per-page/dynamic</t>
-        </is>
-      </c>
-      <c r="G19" t="inlineStr">
+      <c r="E19" s="8" t="inlineStr">
+        <is>
+          <t>Compliant</t>
+        </is>
+      </c>
+      <c r="F19" s="8" t="inlineStr">
+        <is>
+          <t>Footer's "Last Updated" date is no longer a hand-maintained string. vite.config.js now injects the real build/deploy timestamp via a define(__BUILD_DATE__) at build time, and Footer.jsx formats it (e.g. "29 July 2026"). It updates itself automatically on every deploy — no manual editing. Matches standard GIGW practice of a single site-wide "Last Updated On" date (per-page dynamic dates would conflate site content with document metadata, which is already shown separately per document).</t>
+        </is>
+      </c>
+      <c r="G19" s="8" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="H19" t="inlineStr">
+      <c r="H19" s="8" t="inlineStr">
         <is>
           <t>M</t>
         </is>
       </c>
-      <c r="I19" t="inlineStr">
+      <c r="I19" s="8" t="inlineStr">
         <is>
           <t>Footer.jsx</t>
+        </is>
+      </c>
+      <c r="J19" s="8" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: enhance UI and functionality across multiple screens
- Refactor ChangePasswordScreen, ForgotPasswordScreen, and Login components to improve background image handling and accessibility.
- Update CitizenDashboard to integrate semantic search functionality, providing AI-generated answers alongside document results.
- Implement file size validation in UploaderDashboard, alerting users to oversized files and enhancing user experience.
- Add publicSemanticSearch API endpoint for AI-driven document search capabilities.
- Improve code readability and maintainability by restructuring and renaming variables for clarity.
</commit_message>
<xml_diff>
--- a/GIGW_DBIM_Compliance_Tasks.xlsx
+++ b/GIGW_DBIM_Compliance_Tasks.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr codeName="ThisWorkbook"/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="1920" yWindow="1920" windowWidth="17280" windowHeight="8880" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
@@ -36,7 +36,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="10">
+  <fills count="12">
     <fill>
       <patternFill/>
     </fill>
@@ -81,14 +81,24 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00C6EFCE"/>
-        <bgColor rgb="00C6EFCE"/>
+        <fgColor rgb="FFC6EFCE"/>
+        <bgColor rgb="FFC6EFCE"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFEB9C"/>
-        <bgColor rgb="00FFEB9C"/>
+        <fgColor rgb="FFFFEB9C"/>
+        <bgColor rgb="FFFFEB9C"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
       </patternFill>
     </fill>
   </fills>
@@ -104,7 +114,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -115,6 +125,8 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1768,92 +1780,102 @@
       </c>
     </row>
     <row r="20" ht="15.6" customHeight="1">
-      <c r="A20" t="n">
+      <c r="A20" s="10" t="n">
         <v>19</v>
       </c>
-      <c r="B20" t="inlineStr">
+      <c r="B20" s="10" t="inlineStr">
         <is>
           <t>Imagery</t>
         </is>
       </c>
-      <c r="C20" t="inlineStr">
+      <c r="C20" s="10" t="inlineStr">
         <is>
           <t>Enforce image size limits (background/banner &lt;=500KB, thumbnail &lt;=100KB, high-res &lt;=5MB)</t>
         </is>
       </c>
-      <c r="D20" t="inlineStr">
+      <c r="D20" s="10" t="inlineStr">
         <is>
           <t>DBIM 6.1.1, Table 6</t>
         </is>
       </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>Missing</t>
-        </is>
-      </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>No client or server-side validation/compression exists on upload</t>
-        </is>
-      </c>
-      <c r="G20" t="inlineStr">
+      <c r="E20" s="10" t="inlineStr">
+        <is>
+          <t>Compliant</t>
+        </is>
+      </c>
+      <c r="F20" s="10" t="inlineStr">
+        <is>
+          <t>Added a client-side upload size cap across every file input in UploaderDashboard.jsx (main document wizard plus the per-entry chapter/section/schedule/annexure/appendix/forms attachments): oversized files are rejected before upload with a visible error (an alert box for the main wizard, a toast for per-entry attachments), never silently sent. DBIM's own tiers (banner/thumbnail/high-res) are photo-specific and don't map onto a PDF/DOCX document repository, so the closest analogous ceiling - the 5MB "high-res" tier - was applied uniformly to all document uploads instead. The dropzone hint text (previously a stale, unenforced "up to 50 MB") was also corrected to read the real 5MB limit from the same constant, so it can't drift out of sync again. Server-side enforcement is out of scope (backend not in this repo).</t>
+        </is>
+      </c>
+      <c r="G20" s="10" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="H20" t="inlineStr">
+      <c r="H20" s="10" t="inlineStr">
         <is>
           <t>M</t>
         </is>
       </c>
-      <c r="I20" t="inlineStr">
+      <c r="I20" s="10" t="inlineStr">
         <is>
           <t>src/services/pdf.js, upload forms</t>
         </is>
       </c>
+      <c r="J20" s="10" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="15.6" customHeight="1">
-      <c r="A21" t="n">
+      <c r="A21" s="10" t="n">
         <v>20</v>
       </c>
-      <c r="B21" t="inlineStr">
+      <c r="B21" s="10" t="inlineStr">
         <is>
           <t>Imagery</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr">
+      <c r="C21" s="10" t="inlineStr">
         <is>
           <t>Alt text must be meaningful, &lt;=140 characters, and avoid generic terms like 'image of'</t>
         </is>
       </c>
-      <c r="D21" t="inlineStr">
+      <c r="D21" s="10" t="inlineStr">
         <is>
           <t>DBIM 6.1.2</t>
         </is>
       </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>Partial</t>
-        </is>
-      </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>Several non-decorative logo instances use empty alt='' (AdminOtpLogin.jsx:106, AdminOtpLoginScreen.jsx:103, ChangePasswordScreen.jsx:90, ForgotPasswordScreen.jsx:130)</t>
-        </is>
-      </c>
-      <c r="G21" t="inlineStr">
+      <c r="E21" s="10" t="inlineStr">
+        <is>
+          <t>Compliant</t>
+        </is>
+      </c>
+      <c r="F21" s="10" t="inlineStr">
+        <is>
+          <t>Fixed the 4 flagged empty alt='' instances on the haryanaLogo brand image (AdminOtpLogin.jsx, AdminOtpLoginScreen.jsx, ChangePasswordScreen.jsx, ForgotPasswordScreen.jsx), changing them to alt="Haryana Government" - matching the convention already used for the same asset elsewhere (Sidebar.jsx, Topbar.jsx, CitizenDashboard.jsx, Login.jsx). Verified the other empty-alt instances in these same files (the blurred bannerBg full-bleed background image) are correctly decorative and were left as alt='' per WCAG/DBIM - decorative images should be skipped by screen readers, not read aloud.</t>
+        </is>
+      </c>
+      <c r="G21" s="10" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="H21" t="inlineStr">
+      <c r="H21" s="10" t="inlineStr">
         <is>
           <t>S</t>
         </is>
       </c>
-      <c r="I21" t="inlineStr">
+      <c r="I21" s="10" t="inlineStr">
         <is>
           <t>Listed files above</t>
+        </is>
+      </c>
+      <c r="J21" s="10" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -1903,139 +1925,150 @@
       </c>
     </row>
     <row r="23" ht="15.6" customHeight="1">
-      <c r="A23" t="n">
+      <c r="A23" s="10" t="n">
         <v>22</v>
       </c>
-      <c r="B23" t="inlineStr">
+      <c r="B23" s="10" t="inlineStr">
         <is>
           <t>Content</t>
         </is>
       </c>
-      <c r="C23" t="inlineStr">
+      <c r="C23" s="10" t="inlineStr">
         <is>
           <t>Functional bilingual (EN/HI) toggle with proper lang and hreflang attributes</t>
         </is>
       </c>
-      <c r="D23" t="inlineStr">
+      <c r="D23" s="10" t="inlineStr">
         <is>
           <t>DBIM 4.2, 7.5</t>
         </is>
       </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>Partial</t>
-        </is>
-      </c>
-      <c r="F23" t="inlineStr">
-        <is>
-          <t>LanguageToggle.jsx now provides a real site-wide EN/HI switcher with lang-attribute sync, covering Login/Citizen/Uploader/Approver - but AdminDashboard, CSODashboard, NodalOfficerDashboard and AuditorDashboard have zero useTranslation usage, so it isn't fully site-wide yet.</t>
-        </is>
-      </c>
-      <c r="G23" t="inlineStr">
+      <c r="E23" s="10" t="inlineStr">
+        <is>
+          <t>Compliant</t>
+        </is>
+      </c>
+      <c r="F23" s="10" t="inlineStr">
+        <is>
+          <t>Extended useTranslation to the two remaining dashboards: CSODashboard.jsx (Analytics tab, Knowledge Graph tab chrome, MIS Report/audit tab) and AuditorDashboard.jsx (MIS Report, Query History, Compliance Report). Only UI chrome was translated - labels, headings, table headers, buttons, badges, empty states, and the app's own static compliance-certificate copy. Left in English, matching the earlier footer-policy-modal precedent: CSO's large embedded mock dataset of constitutional/legal amendment quotes (NODE_HISTORY) and Knowledge Graph node/link descriptions, and both dashboards' MOCK_AUDIT/MOCK_QUERIES/COMPLIANCE_MONTHS demo data rows (names, actions, queries, numbers) - none of that is real UI copy. Combined with the nodal, admin and footer work already done, every dashboard now has a functional bilingual toggle. Remaining non-dashboard screens (AdminOtpLogin*, ForgotPasswordScreen, ChangePasswordScreen) and the footer's policy-modal content are still English-only by prior explicit scope decisions.</t>
+        </is>
+      </c>
+      <c r="G23" s="10" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="H23" t="inlineStr">
+      <c r="H23" s="10" t="inlineStr">
         <is>
           <t>L</t>
         </is>
       </c>
-      <c r="I23" t="inlineStr">
+      <c r="I23" s="10" t="inlineStr">
         <is>
           <t>App-wide i18n implementation</t>
         </is>
       </c>
+      <c r="J23" s="10" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
     </row>
     <row r="24" ht="15.6" customHeight="1">
-      <c r="A24" t="n">
+      <c r="A24" s="10" t="n">
         <v>23</v>
       </c>
-      <c r="B24" t="inlineStr">
+      <c r="B24" s="10" t="inlineStr">
         <is>
           <t>Content</t>
         </is>
       </c>
-      <c r="C24" t="inlineStr">
+      <c r="C24" s="10" t="inlineStr">
         <is>
           <t>Cookie consent banner (accept/reject/customize) per DPDP Act 2023</t>
         </is>
       </c>
-      <c r="D24" t="inlineStr">
+      <c r="D24" s="10" t="inlineStr">
         <is>
           <t>DBIM 7.6.1, Fig 40-41</t>
         </is>
       </c>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t>Partial</t>
-        </is>
-      </c>
-      <c r="F24" t="inlineStr">
-        <is>
-          <t>src/components/CookieBanner.jsx is a fully-built DPDP-compliant consent banner, but it is never imported/rendered in App.jsx or main.jsx - dead code today; just needs to be mounted.</t>
-        </is>
-      </c>
-      <c r="G24" t="inlineStr">
+      <c r="E24" s="10" t="inlineStr">
+        <is>
+          <t>Compliant</t>
+        </is>
+      </c>
+      <c r="F24" s="10" t="inlineStr">
+        <is>
+          <t>CookieBanner.jsx was already fully built and DPDP-compliant (accept/reject/customise, essential/analytics/functional categories, localStorage-persisted choice) but was dead code - never imported anywhere. Mounted it in App.jsx at every top-level return branch (Login screen, ChangePasswordScreen, the null-activePage frame, and the main authenticated Layout), so it shows on first visit regardless of login state or role. No behavioural changes made to the component itself.</t>
+        </is>
+      </c>
+      <c r="G24" s="10" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="H24" t="inlineStr">
+      <c r="H24" s="10" t="inlineStr">
         <is>
           <t>M</t>
         </is>
       </c>
-      <c r="I24" t="inlineStr">
+      <c r="I24" s="10" t="inlineStr">
         <is>
           <t>src/App.jsx + new CookieConsent component</t>
         </is>
       </c>
+      <c r="J24" s="10" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
     </row>
     <row r="25" ht="15.6" customHeight="1">
-      <c r="A25" t="n">
+      <c r="A25" s="11" t="n">
         <v>24</v>
       </c>
-      <c r="B25" t="inlineStr">
+      <c r="B25" s="11" t="inlineStr">
         <is>
           <t>Content</t>
         </is>
       </c>
-      <c r="C25" t="inlineStr">
+      <c r="C25" s="11" t="inlineStr">
         <is>
           <t>Uploaded documents must be accessible PDFs only, no editable formats</t>
         </is>
       </c>
-      <c r="D25" t="inlineStr">
+      <c r="D25" s="11" t="inlineStr">
         <is>
           <t>DBIM 7.1.3.3</t>
         </is>
       </c>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t>Non-compliant</t>
-        </is>
-      </c>
-      <c r="F25" t="inlineStr">
-        <is>
-          <t>UploaderDashboard.jsx file inputs use accept='.pdf,.doc,.docx' in multiple places - editable Word formats are explicitly accepted, contradicting the PDFs-only requirement.</t>
-        </is>
-      </c>
-      <c r="G25" t="inlineStr">
+      <c r="E25" s="11" t="inlineStr">
+        <is>
+          <t>Non-compliant (by design)</t>
+        </is>
+      </c>
+      <c r="F25" s="11" t="inlineStr">
+        <is>
+          <t>Initially restricted uploads to PDF-only per this guideline (isAccepted() limited to PDF, accept attributes changed to '.pdf', '.DOC' badge and 'PDF or Word' hint removed). Reverted on explicit instruction: the department requires Word (.doc/.docx) upload support as a hard business requirement, which overrides this DBIM clause. UploaderDashboard.jsx now accepts PDF + DOC/DOCX only (isAccepted(), all 4 file inputs' accept attribute, and the per-entry attachment type guards) - everything else is still rejected, so the file-type allowlist stays tight, just wider than DBIM recommends. This is a deliberate, documented business decision, not an oversight - do not re-restrict to PDF-only without checking with the department first.</t>
+        </is>
+      </c>
+      <c r="G25" s="11" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="H25" t="inlineStr">
+      <c r="H25" s="11" t="inlineStr">
         <is>
           <t>M</t>
         </is>
       </c>
-      <c r="I25" t="inlineStr">
+      <c r="I25" s="11" t="inlineStr">
         <is>
           <t>src/pages/UploaderDashboard.jsx, backend</t>
         </is>
       </c>
+      <c r="J25" s="11" t="n"/>
     </row>
     <row r="26" ht="15.6" customHeight="1">
       <c r="A26" t="n">

</xml_diff>

<commit_message>
Update GIGW_DBIM_Compliance_Tasks.xlsx with new compliance data
</commit_message>
<xml_diff>
--- a/GIGW_DBIM_Compliance_Tasks.xlsx
+++ b/GIGW_DBIM_Compliance_Tasks.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr codeName="ThisWorkbook"/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="1920" yWindow="1920" windowWidth="17280" windowHeight="8880" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
@@ -36,7 +36,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="12">
+  <fills count="13">
     <fill>
       <patternFill/>
     </fill>
@@ -101,6 +101,12 @@
         <fgColor rgb="FFFFEB9C"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFD9D9D9"/>
+        <bgColor rgb="FFD9D9D9"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -114,7 +120,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -127,6 +133,7 @@
     <xf numFmtId="0" fontId="0" fillId="9" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="10" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="11" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2071,837 +2078,902 @@
       <c r="J25" s="11" t="n"/>
     </row>
     <row r="26" ht="15.6" customHeight="1">
-      <c r="A26" t="n">
+      <c r="A26" s="8" t="n">
         <v>25</v>
       </c>
-      <c r="B26" t="inlineStr">
+      <c r="B26" s="8" t="inlineStr">
         <is>
           <t>Content</t>
         </is>
       </c>
-      <c r="C26" t="inlineStr">
+      <c r="C26" s="8" t="inlineStr">
         <is>
           <t>Tone of voice: concise, plain language, no Hinglish, uniform British English</t>
         </is>
       </c>
-      <c r="D26" t="inlineStr">
+      <c r="D26" s="8" t="inlineStr">
         <is>
           <t>DBIM 7.1.3</t>
         </is>
       </c>
-      <c r="E26" t="inlineStr">
-        <is>
-          <t>Not audited</t>
-        </is>
-      </c>
-      <c r="F26" t="inlineStr">
-        <is>
-          <t>Needs a dedicated content/copy review pass</t>
-        </is>
-      </c>
-      <c r="G26" t="inlineStr">
+      <c r="E26" s="8" t="inlineStr">
+        <is>
+          <t>Compliant</t>
+        </is>
+      </c>
+      <c r="F26" s="8" t="inlineStr">
+        <is>
+          <t>Audited app-wide UI copy (all src/i18n/locales/en/*.json plus hardcoded JSX text/attributes) for the three DBIM 7.1.3 sub-clauses. No Hinglish found (grep for common roman-script Hindi terms in en/*.json returned nothing). One Americanism found and fixed: pickColor in en/approver.json read "Pick color", corrected to "Pick colour" (uniform British English). Plain-language/conciseness spot-checked across dashboards - labels are already short and direct. Mock/demo data strings (e.g. AuditorDashboard.jsx MOCK_QUERIES) intentionally left untouched, same scope precedent as item 22 - not real UI copy.</t>
+        </is>
+      </c>
+      <c r="G26" s="8" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="H26" t="inlineStr">
+      <c r="H26" s="8" t="inlineStr">
         <is>
           <t>M</t>
         </is>
       </c>
-      <c r="I26" t="inlineStr">
+      <c r="I26" s="8" t="inlineStr">
         <is>
           <t>App-wide UI copy</t>
         </is>
       </c>
+      <c r="J26" s="8" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
     </row>
     <row r="27" ht="15.6" customHeight="1">
-      <c r="A27" t="n">
+      <c r="A27" s="12" t="n">
         <v>26</v>
       </c>
-      <c r="B27" t="inlineStr">
+      <c r="B27" s="12" t="inlineStr">
         <is>
           <t>Content</t>
         </is>
       </c>
-      <c r="C27" t="inlineStr">
+      <c r="C27" s="12" t="inlineStr">
         <is>
           <t>Central Content Publishing System (CCPS) integration for whole-of-government banners/posts</t>
         </is>
       </c>
-      <c r="D27" t="inlineStr">
+      <c r="D27" s="12" t="inlineStr">
         <is>
           <t>DBIM 7.4</t>
         </is>
       </c>
-      <c r="E27" t="inlineStr">
+      <c r="E27" s="12" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="F27" t="inlineStr">
+      <c r="F27" s="12" t="inlineStr">
         <is>
           <t>CCPS is a Central Ministry/MeitY system; not applicable to a State department portal</t>
         </is>
       </c>
-      <c r="G27" t="inlineStr">
+      <c r="G27" s="12" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="H27" t="inlineStr">
+      <c r="H27" s="12" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="I27" t="inlineStr">
+      <c r="I27" s="12" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
+      <c r="J27" s="12" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
     </row>
     <row r="28" ht="15.6" customHeight="1">
-      <c r="A28" t="n">
+      <c r="A28" s="8" t="n">
         <v>27</v>
       </c>
-      <c r="B28" t="inlineStr">
+      <c r="B28" s="8" t="inlineStr">
         <is>
           <t>Accessibility</t>
         </is>
       </c>
-      <c r="C28" t="inlineStr">
+      <c r="C28" s="8" t="inlineStr">
         <is>
           <t>Activate skip-to-main-content link</t>
         </is>
       </c>
-      <c r="D28" t="inlineStr">
+      <c r="D28" s="8" t="inlineStr">
         <is>
           <t>GIGW / DBIM 8.2</t>
         </is>
       </c>
-      <c r="E28" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="F28" t="inlineStr">
+      <c r="E28" s="8" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F28" s="8" t="inlineStr">
         <is>
           <t>CSS for .skip-nav exists but sits inside a disabled comment block labelled 'DBIM / GIGW compliance - enable in production'; no &lt;a&gt; element renders it</t>
         </is>
       </c>
-      <c r="G28" t="inlineStr">
+      <c r="G28" s="8" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="H28" t="inlineStr">
+      <c r="H28" s="8" t="inlineStr">
         <is>
           <t>S</t>
         </is>
       </c>
-      <c r="I28" t="inlineStr">
+      <c r="I28" s="8" t="inlineStr">
         <is>
           <t>src/index.css:141-180, src/components/layout/Layout.jsx</t>
         </is>
       </c>
-      <c r="J28" s="1" t="inlineStr">
+      <c r="J28" s="8" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
     <row r="29" ht="15.6" customHeight="1">
-      <c r="A29" t="n">
+      <c r="A29" s="8" t="n">
         <v>28</v>
       </c>
-      <c r="B29" t="inlineStr">
+      <c r="B29" s="8" t="inlineStr">
         <is>
           <t>Accessibility</t>
         </is>
       </c>
-      <c r="C29" t="inlineStr">
+      <c r="C29" s="8" t="inlineStr">
         <is>
           <t>Text-size adjuster (A+ / A-)</t>
         </is>
       </c>
-      <c r="D29" t="inlineStr">
+      <c r="D29" s="8" t="inlineStr">
         <is>
           <t>GIGW / DBIM Fig 44</t>
         </is>
       </c>
-      <c r="E29" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="F29" t="inlineStr">
+      <c r="E29" s="8" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F29" s="8" t="inlineStr">
         <is>
           <t>CSS (html[data-font-size]) exists but no UI control is wired to it</t>
         </is>
       </c>
-      <c r="G29" t="inlineStr">
+      <c r="G29" s="8" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="H29" t="inlineStr">
+      <c r="H29" s="8" t="inlineStr">
         <is>
           <t>M</t>
         </is>
       </c>
-      <c r="I29" t="inlineStr">
+      <c r="I29" s="8" t="inlineStr">
         <is>
           <t>Topbar.jsx + index.css</t>
         </is>
       </c>
-      <c r="J29" s="1" t="inlineStr">
+      <c r="J29" s="8" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
     <row r="30" ht="15.6" customHeight="1">
-      <c r="A30" t="n">
+      <c r="A30" s="8" t="n">
         <v>29</v>
       </c>
-      <c r="B30" t="inlineStr">
+      <c r="B30" s="8" t="inlineStr">
         <is>
           <t>Accessibility</t>
         </is>
       </c>
-      <c r="C30" t="inlineStr">
+      <c r="C30" s="8" t="inlineStr">
         <is>
           <t>High-contrast mode toggle</t>
         </is>
       </c>
-      <c r="D30" t="inlineStr">
+      <c r="D30" s="8" t="inlineStr">
         <is>
           <t>GIGW / DBIM Fig 44</t>
         </is>
       </c>
-      <c r="E30" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="F30" t="inlineStr">
+      <c r="E30" s="8" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F30" s="8" t="inlineStr">
         <is>
           <t>CSS (html[data-contrast="high"]) exists but no UI control is wired to it</t>
         </is>
       </c>
-      <c r="G30" t="inlineStr">
+      <c r="G30" s="8" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="H30" t="inlineStr">
+      <c r="H30" s="8" t="inlineStr">
         <is>
           <t>M</t>
         </is>
       </c>
-      <c r="I30" t="inlineStr">
+      <c r="I30" s="8" t="inlineStr">
         <is>
           <t>Topbar.jsx + index.css</t>
         </is>
       </c>
-      <c r="J30" s="1" t="inlineStr">
+      <c r="J30" s="8" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
     <row r="31" ht="15.6" customHeight="1">
-      <c r="A31" t="n">
+      <c r="A31" s="8" t="n">
         <v>30</v>
       </c>
-      <c r="B31" t="inlineStr">
+      <c r="B31" s="8" t="inlineStr">
         <is>
           <t>Accessibility</t>
         </is>
       </c>
-      <c r="C31" t="inlineStr">
+      <c r="C31" s="8" t="inlineStr">
         <is>
           <t>Real Screen Reader Access / Accessibility Statement page</t>
         </is>
       </c>
-      <c r="D31" t="inlineStr">
+      <c r="D31" s="8" t="inlineStr">
         <is>
           <t>GIGW</t>
         </is>
       </c>
-      <c r="E31" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="F31" t="inlineStr">
+      <c r="E31" s="8" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F31" s="8" t="inlineStr">
         <is>
           <t>Footer.jsx:15 links to an anchor stub (href='#screen-reader'), not a real page</t>
         </is>
       </c>
-      <c r="G31" t="inlineStr">
+      <c r="G31" s="8" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="H31" t="inlineStr">
+      <c r="H31" s="8" t="inlineStr">
         <is>
           <t>S</t>
         </is>
       </c>
-      <c r="I31" t="inlineStr">
+      <c r="I31" s="8" t="inlineStr">
         <is>
           <t>New page + Footer.jsx</t>
         </is>
       </c>
-      <c r="J31" s="1" t="inlineStr">
+      <c r="J31" s="8" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
     <row r="32" ht="15.6" customHeight="1">
-      <c r="A32" t="n">
+      <c r="A32" s="8" t="n">
         <v>31</v>
       </c>
-      <c r="B32" t="inlineStr">
+      <c r="B32" s="8" t="inlineStr">
         <is>
           <t>Accessibility</t>
         </is>
       </c>
-      <c r="C32" t="inlineStr">
+      <c r="C32" s="8" t="inlineStr">
         <is>
           <t>Consistent &lt;label htmlFor&gt; bindings on all form inputs</t>
         </is>
       </c>
-      <c r="D32" t="inlineStr">
+      <c r="D32" s="8" t="inlineStr">
         <is>
           <t>GIGW / DBIM Annexure B</t>
         </is>
       </c>
-      <c r="E32" t="inlineStr">
+      <c r="E32" s="8" t="inlineStr">
+        <is>
+          <t>Compliant</t>
+        </is>
+      </c>
+      <c r="F32" s="8" t="inlineStr">
+        <is>
+          <t>Wired id/htmlFor pairs across every remaining unlabeled form input app-wide: Login.jsx (2), AdminDashboard.jsx (17: add-user drawer, edit-user modal, add-department modal), NodalOfficerDashboard.jsx (12 of 13 - the 13th is a read-only role display div in the edit modal, not a focusable control, so no htmlFor target exists), AdminOtpLogin.jsx + AdminOtpLoginScreen.jsx (2+2), ChangePasswordScreen.jsx (3) and ForgotPasswordScreen.jsx (4). Extended the shared SelectField.jsx and AdminDashboard.jsx-local MultiSelectField (custom button-triggered dropdowns, not native &lt;select&gt;) to accept an id prop applied to their trigger button, so htmlFor still resolves correctly on those. UploaderDashboard.jsx checkbox labels already used the valid implicit wrap pattern (&lt;label&gt;&lt;input type=checkbox/&gt;text&lt;/label&gt;) - no change needed there. Also fixed a stricter form of the same gap: ApproverDashboard.jsx (5) and CSODashboard.jsx (2) had inputs with no &lt;label&gt; at all (icon-only search boxes, an annotation-comment textarea, numbered remark fields) - added real &lt;label htmlFor&gt; where a visible caption already existed, and aria-label on the two icon-only search boxes where adding a visible label would require a layout change. Verified with npx vite build (clean) and npx eslint (no new errors - all pre-existing lint findings are unrelated setState-in-effect/unused-var issues, none on touched lines).</t>
+        </is>
+      </c>
+      <c r="G32" s="8" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H32" s="8" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="I32" s="8" t="inlineStr">
+        <is>
+          <t>All form components</t>
+        </is>
+      </c>
+      <c r="J32" s="8" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="15.6" customHeight="1">
+      <c r="A33" s="8" t="n">
+        <v>32</v>
+      </c>
+      <c r="B33" s="8" t="inlineStr">
+        <is>
+          <t>Accessibility</t>
+        </is>
+      </c>
+      <c r="C33" s="8" t="inlineStr">
+        <is>
+          <t>Keyboard navigability with a visible focus-visible state</t>
+        </is>
+      </c>
+      <c r="D33" s="8" t="inlineStr">
+        <is>
+          <t>GIGW / DBIM 8.2</t>
+        </is>
+      </c>
+      <c r="E33" s="8" t="inlineStr">
+        <is>
+          <t>Compliant</t>
+        </is>
+      </c>
+      <c r="F33" s="8" t="inlineStr">
+        <is>
+          <t>Old note was stale (claimed zero tabIndex usage) - a global :focus-visible rule with !important already existed (index.css:235, from item 9) and UploaderDashboard.jsx already had 4 correctly keyboard-operable custom controls. But the real requirement - every custom clickable control being keyboard-reachable - had 11 genuine violations: plain &lt;div onClick&gt; with no role/tabIndex/onKeyDown, found via a repo-wide audit (excluding modal-backdrop/stopPropagation wrappers, which do not need keyboard access). Fixed all 11: Login.jsx (3 portal-selection cards - the critical role-picker on the app front door - plus the password show/hide toggle), ChangePasswordScreen.jsx and ForgotPasswordScreen.jsx password toggles, ProfileModal.jsx password toggle, Topbar.jsx profile-menu items (Edit Profile / Logout), ApproverDashboard.jsx (annotation-list item, doc-row expand/collapse), CSODashboard.jsx (graph node-selector chip), and the shared Card.jsx component (adds role/tabIndex/onKeyDown automatically whenever an onClick prop is passed, fixing 5 more call sites app-wide in one place: AdminDashboard stat filters, ApproverDashboard nav/filter cards, UploaderDashboard action cards). Added showPassword/hidePassword i18n keys to login.json (en+hi) for the one screen that uses i18n; other auth screens use plain string aria-labels per their existing English-only scope. Verified: npx vite build clean, npx eslint shows no new issues (all remaining findings are pre-existing, unrelated setState-in-effect/unused-var patterns).</t>
+        </is>
+      </c>
+      <c r="G33" s="8" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H33" s="8" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="I33" s="8" t="inlineStr">
+        <is>
+          <t>src/index.css</t>
+        </is>
+      </c>
+      <c r="J33" s="8" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="15.6" customHeight="1">
+      <c r="A34" s="8" t="n">
+        <v>33</v>
+      </c>
+      <c r="B34" s="8" t="inlineStr">
+        <is>
+          <t>Accessibility</t>
+        </is>
+      </c>
+      <c r="C34" s="8" t="inlineStr">
+        <is>
+          <t>Colour contrast for text over the selected palette</t>
+        </is>
+      </c>
+      <c r="D34" s="8" t="inlineStr">
+        <is>
+          <t>GIGW / DBIM 4.4</t>
+        </is>
+      </c>
+      <c r="E34" s="8" t="inlineStr">
+        <is>
+          <t>Compliant</t>
+        </is>
+      </c>
+      <c r="F34" s="8" t="inlineStr">
+        <is>
+          <t>Re-ran contrast checks now that the palette (items 1/3) is finalized. Computed real WCAG 2.1 contrast ratios (relative-luminance formula) for every text/background pair actually used in index.css, plus the real composited Badge.jsx colours (not just the raw CSS vars in isolation): body text, headings, primary buttons/links, footer text on primary-dark, and all 4 status-colour badges all pass AA (4.5-20:1). High-contrast mode pairs all pass with large margin (9-17:1). Found one genuine but marginal failure: --text-color-secondary (#6c757d) directly on --surface-ground (#f8f9fa) measured 4.45:1, just under the 4.5:1 AA threshold - this var backs the small uppercase LABEL style duplicated across nearly every dashboard file for field labels/table headers. Fixed by nudging it to #6b747c in index.css:109 (1 unit per RGB channel, visually imperceptible) - re-verified both worst-case pairs now pass: 4.51:1 on surface-ground, 4.76:1 on surface-card. Also noted --amber (#FFC107) fails badly in isolation (1.63:1) but is never consumed directly in any JSX (Badge.jsx uses its own separate accessible dark-on-tint amber pair instead), so it is a dead/unused CSS token, not a live on-screen bug. Verified with npx vite build (clean).</t>
+        </is>
+      </c>
+      <c r="G34" s="8" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H34" s="8" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="I34" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J34" s="8" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="15.6" customHeight="1">
+      <c r="A35" s="12" t="n">
+        <v>34</v>
+      </c>
+      <c r="B35" s="12" t="inlineStr">
+        <is>
+          <t>Search</t>
+        </is>
+      </c>
+      <c r="C35" s="12" t="inlineStr">
+        <is>
+          <t>Enhanced search: multi-language, filtered/categorized results, autocomplete, spell correction, covers PDFs/HTML/metadata</t>
+        </is>
+      </c>
+      <c r="D35" s="12" t="inlineStr">
+        <is>
+          <t>DBIM 9</t>
+        </is>
+      </c>
+      <c r="E35" s="12" t="inlineStr">
         <is>
           <t>Partial</t>
         </is>
       </c>
-      <c r="F32" t="inlineStr">
-        <is>
-          <t>Login.jsx uses proper labels; Uploader/Admin forms rely on placeholder text only - zero htmlFor usage found app-wide</t>
-        </is>
-      </c>
-      <c r="G32" t="inlineStr">
+      <c r="F35" s="12" t="inlineStr">
+        <is>
+          <t>DONE already (verified in code, CitizenDashboard.jsx): (1) Autocomplete - debounced live-suggestions dropdown (line ~297-308) hitting /pdf/public/search as you type, shows real matching documents with highlighted text. (2) Category filter - document-type dropdown (line ~561) filters both autocomplete and main search. (3) Semantic/AI search - the Search button calls /pdf/public/semantic-search (services/pdf.js:20), meaning-based matching, not just literal keywords - this already gives some natural typo-tolerance for free. STILL REMAINING (all backend/search-index work, outside this frontend repo, so unverifiable/unbuildable from here - do NOT attempt to fake these client-side): (a) Explicit spell-correction ('did you mean...') - needs a backend fuzzy-match layer (e.g. Elasticsearch/OpenSearch suggester, or a Levenshtein-based re-ranker) on top of /pdf/public/search. (b) Multi-language search verification - need to confirm a Hindi-script query against /pdf/public/semantic-search actually returns correct results (requires the backend embedding model to be multilingual) - untested because backend is not in this repo; test this once a backend/dev server is available. (c) Confirm search actually indexes PDF body content + metadata (department, year, act name) and not just filename/document_name - check the backend indexing pipeline, not frontend code. (d) Only ONE filter facet exists today (document type) - DBIM 9 implies richer filtering (department, year, language); if /pdf/public/search already accepts extra params like department_id server-side, wiring more filter UI here would be a quick frontend-only win - confirm with backend team what params the endpoint actually supports before adding UI for them. Next step when picking this back up: get backend/API access, verify (b) and (c) first since they determine whether (a) and (d) are even worth doing.</t>
+        </is>
+      </c>
+      <c r="G35" s="12" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="H32" t="inlineStr">
+      <c r="H35" s="12" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="I35" s="12" t="inlineStr">
+        <is>
+          <t>Search feature + backend</t>
+        </is>
+      </c>
+      <c r="J35" s="12" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="15.6" customHeight="1">
+      <c r="A36" s="12" t="n">
+        <v>35</v>
+      </c>
+      <c r="B36" s="12" t="inlineStr">
+        <is>
+          <t>Search</t>
+        </is>
+      </c>
+      <c r="C36" s="12" t="inlineStr">
+        <is>
+          <t>Consistent search box placement in the header across all pages</t>
+        </is>
+      </c>
+      <c r="D36" s="12" t="inlineStr">
+        <is>
+          <t>DBIM 9(v)</t>
+        </is>
+      </c>
+      <c r="E36" s="12" t="inlineStr">
+        <is>
+          <t>Non-compliant (by design)</t>
+        </is>
+      </c>
+      <c r="F36" s="12" t="inlineStr">
+        <is>
+          <t>Accepted as an intentional trade-off, same reasoning as item #9/12's decision: a generic global search box has no clear target in an internal staff tool (Admin/Approver/Uploader/Nodal/CSO) - each already has its own scoped, in-page table-filter search relevant to that screen's data. The Citizen Dashboard, which is the actual public-facing page DBIM 9(v) is aimed at, already has a real header-docked search bar. Forcing an identical header search box onto every staff dashboard would just be visual consistency for its own sake, not a real usability improvement, and was rejected on that basis. IF THIS DECISION IS EVER REVISITED, changes needed to become fully compliant: (1) Add a search input to the shared Topbar.jsx (src/components/layout/Topbar.jsx) so it renders in the same position on every staff dashboard, not just Citizen. (2) Decide what it should actually search - either (a) make it a no-op/decorative element purely for layout consistency (not recommended - a search box that doesn't search is worse UX), or (b) wire it to each page's existing local filter state (searchQ/auditSearch/etc. - already present per-dashboard, see item #34's notes) so the header box becomes the single source of truth instead of the current in-page boxes, which would also require removing/consolidating the existing per-page search inputs so there isn't a confusing duplicate search box on screen at once. (3) Re-test keyboard/i18n/RTL behaviour of the new shared header search across all 5 staff dashboards.</t>
+        </is>
+      </c>
+      <c r="G36" s="12" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H36" s="12" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="I36" s="12" t="inlineStr">
+        <is>
+          <t>Topbar.jsx</t>
+        </is>
+      </c>
+      <c r="J36" s="12" t="inlineStr">
+        <is>
+          <t>Accepted</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="15.6" customHeight="1">
+      <c r="A37" s="8" t="n">
+        <v>36</v>
+      </c>
+      <c r="B37" s="8" t="inlineStr">
+        <is>
+          <t>Performance</t>
+        </is>
+      </c>
+      <c r="C37" s="8" t="inlineStr">
+        <is>
+          <t>Lazy-load images and media</t>
+        </is>
+      </c>
+      <c r="D37" s="8" t="inlineStr">
+        <is>
+          <t>DBIM 10.1.2</t>
+        </is>
+      </c>
+      <c r="E37" s="8" t="inlineStr">
+        <is>
+          <t>Compliant</t>
+        </is>
+      </c>
+      <c r="F37" s="8" t="inlineStr">
+        <is>
+          <t>Audited all 18 &lt;img&gt; tags app-wide. Found every single one is either a persistent header/footer logo (Haryana logo, Ashoka emblem, Digital India logo) or a full-screen hero background (bannerBg) - there are currently no below-the-fold/offscreen images anywhere in the app (no document-thumbnail galleries, no long image feeds), so real lazy-loading has nothing to save yet. Added loading='lazy' to the 12 small logo images (Footer.jsx x2, Sidebar.jsx, Topbar.jsx, AdminOtpLogin.jsx, AdminOtpLoginScreen.jsx, ChangePasswordScreen.jsx, ForgotPasswordScreen.jsx, CitizenDashboard.jsx x2, Login.jsx x2) - satisfies the literal requirement and is harmless since browsers still eagerly load anything already in the initial viewport regardless of the lazy hint. Deliberately did NOT add it to the 6 bannerBg hero images (Login.jsx x2, AdminOtpLogin.jsx, ChangePasswordScreen.jsx, ForgotPasswordScreen.jsx, CitizenDashboard.jsx) - each is that page's LCP (largest contentful paint) candidate, and lazy-loading the LCP image is an explicitly discouraged anti-pattern (Lighthouse flags it) since it would delay the very metric this performance category is meant to protect. If real content images are added later (e.g. a document thumbnail gallery), apply loading='lazy' to those too. Verified with npx vite build (clean).</t>
+        </is>
+      </c>
+      <c r="G37" s="8" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H37" s="8" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="I37" s="8" t="inlineStr">
+        <is>
+          <t>App-wide</t>
+        </is>
+      </c>
+      <c r="J37" s="8" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="15.6" customHeight="1">
+      <c r="A38" s="12" t="n">
+        <v>37</v>
+      </c>
+      <c r="B38" s="12" t="inlineStr">
+        <is>
+          <t>Performance</t>
+        </is>
+      </c>
+      <c r="C38" s="12" t="inlineStr">
+        <is>
+          <t>Image compression/optimization pipeline before publishing</t>
+        </is>
+      </c>
+      <c r="D38" s="12" t="inlineStr">
+        <is>
+          <t>DBIM 10.3.2</t>
+        </is>
+      </c>
+      <c r="E38" s="12" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="F38" s="12" t="inlineStr">
+        <is>
+          <t>Old note was stale (said 'Upload backend' - wrong, this app only accepts PDF/DOC/DOCX uploads per item #24, never raw images, so there is no upload-side image pipeline to build). The real target is the app's own bundled assets in src/assets/. Measured actual compression potential (Pillow re-encode test) on the 2 raster assets: banner-1-768x217.png (120.3KB, used as the full-screen hero background on 6 screens: Login x2, AdminOtpLogin, ChangePasswordScreen, ForgotPasswordScreen, CitizenDashboard) - converting to WebP q82 measured 43.2KB, a real 64% reduction, no visible quality loss (it is a blurred/covered background). haryana-logo.png (31.0KB, small header/footer logo) - PNG re-optimize and WebP both made it BIGGER (36.9KB / 68.5KB) - has transparency/sharp edges lossy formats handle poorly, so leave as plain PNG. NOT YET DONE (paused here on explicit instruction, revisit later): (1) Convert banner-1-768x217.png to .webp and update the bannerBg import path in the 5 files that use it, delete the old PNG - biggest win, ~77KB saved on first paint of 6 screens. (2) Optionally add a real build-time image-optimization pipeline (e.g. an imagemin-based Vite plugin) so future images added by any dev get auto-compressed at build time, not just this one manual fix - not attempted yet because this repo runs Vite 8 (bleeding-edge rolldown-vite) and third-party imagemin plugins use native binaries that may not be compatible; test compatibility in a throwaway branch first before adding as a real dependency. (3) Do NOT touch haryana-logo.png - confirmed no format gives a real size reduction for it.</t>
+        </is>
+      </c>
+      <c r="G38" s="12" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H38" s="12" t="inlineStr">
         <is>
           <t>M</t>
         </is>
       </c>
-      <c r="I32" t="inlineStr">
-        <is>
-          <t>All form components</t>
-        </is>
-      </c>
-    </row>
-    <row r="33" ht="15.6" customHeight="1">
-      <c r="A33" t="n">
-        <v>32</v>
-      </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>Accessibility</t>
-        </is>
-      </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>Keyboard navigability with a visible focus-visible state</t>
-        </is>
-      </c>
-      <c r="D33" t="inlineStr">
-        <is>
-          <t>GIGW / DBIM 8.2</t>
-        </is>
-      </c>
-      <c r="E33" t="inlineStr">
+      <c r="I38" s="12" t="inlineStr">
+        <is>
+          <t>Upload backend</t>
+        </is>
+      </c>
+      <c r="J38" s="12" t="inlineStr">
         <is>
           <t>Partial</t>
         </is>
       </c>
-      <c r="F33" t="inlineStr">
-        <is>
-          <t>Some :focus styles exist but there is no global focus-visible strategy; zero tabIndex usage found</t>
-        </is>
-      </c>
-      <c r="G33" t="inlineStr">
+    </row>
+    <row r="39" ht="15.6" customHeight="1">
+      <c r="A39" s="9" t="n">
+        <v>38</v>
+      </c>
+      <c r="B39" s="9" t="inlineStr">
+        <is>
+          <t>Performance</t>
+        </is>
+      </c>
+      <c r="C39" s="9" t="inlineStr">
+        <is>
+          <t>Analytics integration (visitor tracking, KPIs, traffic dashboard)</t>
+        </is>
+      </c>
+      <c r="D39" s="9" t="inlineStr">
+        <is>
+          <t>DBIM 10.5-10.6</t>
+        </is>
+      </c>
+      <c r="E39" s="9" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="F39" s="9" t="inlineStr">
+        <is>
+          <t>CSODashboard.jsx Analytics tab already shows real document KPIs (totals, dept breakdown, status distribution, monthly trend) - that part is done. What's missing is real VISITOR/TRAFFIC analytics (unique visitors, page views, session duration) - genuinely blocked, not on code but on missing infrastructure: this needs an actual analytics account/property (Google Analytics 4, Matomo, Plausible, or a self-hosted visitor-counter backend endpoint) that someone in the department has to create first. Do NOT wire in a placeholder/fake tracking ID just to look done - a fake G-XXXXXXX in index.html would silently send data nowhere, which is worse than leaving this honestly incomplete. TO MAKE THIS COMPLIANT LATER: (1) Get a real analytics account provisioned - either ask IT/department for a GA4 property ID, or spin up a self-hosted option (Matomo/Plausible) if data-privacy rules prefer not sending citizen traffic data to Google. (2) Once a real tracking ID/script snippet exists, add it to index.html (or src/main.jsx as a lazy-loaded script) - this part really is a 10-minute job once step 1 is done. (3) Surface the resulting visitor/traffic numbers somewhere in CSODashboard's Analytics tab alongside the existing document KPIs, so this becomes one unified analytics view instead of two separate things.</t>
+        </is>
+      </c>
+      <c r="G39" s="9" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H39" s="9" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="I39" s="9" t="inlineStr">
+        <is>
+          <t>index.html / src/main.jsx</t>
+        </is>
+      </c>
+      <c r="J39" s="9" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="15.6" customHeight="1">
+      <c r="A40" s="9" t="n">
+        <v>39</v>
+      </c>
+      <c r="B40" s="9" t="inlineStr">
+        <is>
+          <t>Forms</t>
+        </is>
+      </c>
+      <c r="C40" s="9" t="inlineStr">
+        <is>
+          <t>Mandatory fields marked with * or "Required"; single-column vertical layout; clickable labels; keyboard-friendly</t>
+        </is>
+      </c>
+      <c r="D40" s="9" t="inlineStr">
+        <is>
+          <t>DBIM Annexure B</t>
+        </is>
+      </c>
+      <c r="E40" s="9" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="F40" s="9" t="inlineStr">
+        <is>
+          <t>4 sub-clauses, 3 now done: 'clickable labels' and 'keyboard-friendly' were already fixed by items #31/#32's htmlFor + keyboard-nav work this session. 'Mandatory fields marked with *' - fixed now: added a red '*' next to the label of every field actually enforced as required in its own validation code (not guessed) - AdminDashboard.jsx Add User (username, email, password) and Add Department (name), NodalOfficerDashboard.jsx Add User (username, email, password, department). Fields with no enforced required-check (first/last name, mobile, role, department in Admin's non-nodal path, Edit User modal - which has no required-field validation at all) were deliberately left unmarked, since marking them '*' would misrepresent what the code actually enforces. STILL NOT DONE (explicit user call this session - marker-only fix requested, layout left alone): 'single-column vertical layout' - both Add User drawers still use a 2-column grid (gridTemplateColumns: '1fr 1fr') for Username+Email and First+Last name pairs, which is a real, structural violation of this clause, not yet addressed. To close this fully, someone needs to decide whether to convert those grids to single-column (will make the Add User drawer noticeably taller/more scrolly - a real visual trade-off, similar to the deliberate call already made on item #8).</t>
+        </is>
+      </c>
+      <c r="G40" s="9" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="H33" t="inlineStr">
-        <is>
-          <t>S</t>
-        </is>
-      </c>
-      <c r="I33" t="inlineStr">
-        <is>
-          <t>src/index.css</t>
-        </is>
-      </c>
-    </row>
-    <row r="34" ht="15.6" customHeight="1">
-      <c r="A34" t="n">
-        <v>33</v>
-      </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>Accessibility</t>
-        </is>
-      </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>Colour contrast for text over the selected palette</t>
-        </is>
-      </c>
-      <c r="D34" t="inlineStr">
-        <is>
-          <t>GIGW / DBIM 4.4</t>
-        </is>
-      </c>
-      <c r="E34" t="inlineStr">
-        <is>
-          <t>Not verified</t>
-        </is>
-      </c>
-      <c r="F34" t="inlineStr">
-        <is>
-          <t>Re-run contrast checks once palette (item 1/3) is finalized</t>
-        </is>
-      </c>
-      <c r="G34" t="inlineStr">
+      <c r="H40" s="9" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="I40" s="9" t="inlineStr">
+        <is>
+          <t>Form components across Admin/Uploader/Nodal dashboards</t>
+        </is>
+      </c>
+      <c r="J40" s="9" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="15.6" customHeight="1">
+      <c r="A41" s="8" t="n">
+        <v>40</v>
+      </c>
+      <c r="B41" s="8" t="inlineStr">
+        <is>
+          <t>Forms</t>
+        </is>
+      </c>
+      <c r="C41" s="8" t="inlineStr">
+        <is>
+          <t>Primary action buttons disabled until required fields are valid, with submit-progress feedback</t>
+        </is>
+      </c>
+      <c r="D41" s="8" t="inlineStr">
+        <is>
+          <t>DBIM Annexure B(xiv)</t>
+        </is>
+      </c>
+      <c r="E41" s="8" t="inlineStr">
+        <is>
+          <t>Compliant</t>
+        </is>
+      </c>
+      <c r="F41" s="8" t="inlineStr">
+        <is>
+          <t>Went app-wide per explicit instruction. Found and fixed the real gap: buttons already showed a spinner 'looks disabled' style while a form was invalid (via an unused canSubmit-style variable) but the actual HTML disabled attribute only checked submit-in-progress, not field validity - meaning invalid forms were still clickable despite looking disabled. Fixed disabled={} to genuinely gate on both submitting AND required-field validity in: AdminDashboard.jsx (Add User: username/email/password; Add Department: name; Edit User: email), NodalOfficerDashboard.jsx (same + department for Add User; email for Edit User), Login.jsx (username/password), AdminOtpLogin.jsx + AdminOtpLoginScreen.jsx (10-digit mobile for step 1, captcha+6-digit OTP for step 2), ChangePasswordScreen.jsx (current password, new password &gt;=8 chars, matching confirm), ForgotPasswordScreen.jsx (identifier for step 1; OTP+new password+match for step 2), UploaderDashboard.jsx Edit Document modal (document_name). ApproverDashboard.jsx: found ThreePanelReview's Reject button had NO comment-required gate even though the sibling LinkReviewPanel already correctly required at least one remark before rejecting - added the same hasRemarks gate + tooltip (new i18n key common.enterRemarkBeforeRejecting, en+hi) so both reject flows are now consistent. The actParts confirm/reject modal was already correctly gated - no change needed there. UploaderDashboard.jsx's main upload wizard, legal-authority/relation-add forms were already properly gated (file-selection / act-selection / target-selection required) - left as-is. Sub-document chapter/section forms use a deliberate dirty-check gate (disabled unless changed) rather than a required-name check, since section/chapter names are legitimately editable as empty drafts - not changed, this is intentional not a gap. Verified with npx vite build (clean) and npx eslint (no new errors - all remaining findings are pre-existing, unrelated setState-in-effect/unused-var issues).</t>
+        </is>
+      </c>
+      <c r="G41" s="8" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H41" s="8" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="I41" s="8" t="inlineStr">
+        <is>
+          <t>Form components app-wide</t>
+        </is>
+      </c>
+      <c r="J41" s="8" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="15.6" customHeight="1">
+      <c r="A42" s="8" t="n">
+        <v>41</v>
+      </c>
+      <c r="B42" s="8" t="inlineStr">
+        <is>
+          <t>Security</t>
+        </is>
+      </c>
+      <c r="C42" s="8" t="inlineStr">
+        <is>
+          <t>CAPTCHA on login/OTP/forgot-password forms</t>
+        </is>
+      </c>
+      <c r="D42" s="8" t="inlineStr">
+        <is>
+          <t>GIGW security baseline</t>
+        </is>
+      </c>
+      <c r="E42" s="8" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F42" s="8" t="inlineStr">
+        <is>
+          <t>No CAPTCHA found on any authentication form</t>
+        </is>
+      </c>
+      <c r="G42" s="8" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H42" s="8" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="I42" s="8" t="inlineStr">
+        <is>
+          <t>src/pages/Login.jsx, AdminOtpLogin*, ForgotPasswordScreen.jsx</t>
+        </is>
+      </c>
+      <c r="J42" s="8" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="15.6" customHeight="1">
+      <c r="A43" s="8" t="n">
+        <v>42</v>
+      </c>
+      <c r="B43" s="8" t="inlineStr">
+        <is>
+          <t>Security</t>
+        </is>
+      </c>
+      <c r="C43" s="8" t="inlineStr">
+        <is>
+          <t>Idle/inactivity session timeout (not just reactive 401 logout)</t>
+        </is>
+      </c>
+      <c r="D43" s="8" t="inlineStr">
+        <is>
+          <t>GIGW</t>
+        </is>
+      </c>
+      <c r="E43" s="8" t="inlineStr">
+        <is>
+          <t>Compliant</t>
+        </is>
+      </c>
+      <c r="F43" s="8" t="inlineStr">
+        <is>
+          <t>Added a real client-side idle timer in src/hooks/useAuth.js, separate from the existing reactive 401-on-expiry handler (services/api.js:17) - the two solve different problems: token expiry ends the session after a fixed lifetime regardless of activity, idle timeout ends it after 15 minutes of no activity even if the token is still valid, protecting an unattended/walked-away-from screen. Listens for mousemove/mousedown/keydown/scroll/touchstart/click on window, resets a 15-minute timer on each event, calls the existing logout() (which already clears the token and notifies the backend) if the timer fires. Only active for real authenticated sessions (gated on user &amp;&amp; role !== 'citizen') - the citizen guest role has no backend session/token to protect, so it's exempt by design. 15 minutes was chosen as a standard government-portal default: this is a policy call, not a technical constraint - adjust IDLE_TIMEOUT_MS in useAuth.js if the department wants a different threshold. Note: this implements the core requirement (auto-logout on inactivity) but not a warning/countdown toast before logout - that would be a nice UX addition for later, not attempted here to keep scope tight to the literal requirement. Verified with npx vite build and npx eslint (both clean, no warnings).</t>
+        </is>
+      </c>
+      <c r="G43" s="8" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="H34" t="inlineStr">
-        <is>
-          <t>S</t>
-        </is>
-      </c>
-      <c r="I34" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="35" ht="15.6" customHeight="1">
-      <c r="A35" t="n">
-        <v>34</v>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>Search</t>
-        </is>
-      </c>
-      <c r="C35" t="inlineStr">
-        <is>
-          <t>Enhanced search: multi-language, filtered/categorized results, autocomplete, spell correction, covers PDFs/HTML/metadata</t>
-        </is>
-      </c>
-      <c r="D35" t="inlineStr">
-        <is>
-          <t>DBIM 9</t>
-        </is>
-      </c>
-      <c r="E35" t="inlineStr">
-        <is>
-          <t>Partial</t>
-        </is>
-      </c>
-      <c r="F35" t="inlineStr">
-        <is>
-          <t>Existing search covers basic keyword matching only; no autocomplete, spell-correction or persona/category filters</t>
-        </is>
-      </c>
-      <c r="G35" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="H35" t="inlineStr">
-        <is>
-          <t>L</t>
-        </is>
-      </c>
-      <c r="I35" t="inlineStr">
-        <is>
-          <t>Search feature + backend</t>
-        </is>
-      </c>
-    </row>
-    <row r="36" ht="15.6" customHeight="1">
-      <c r="A36" t="n">
-        <v>35</v>
-      </c>
-      <c r="B36" t="inlineStr">
-        <is>
-          <t>Search</t>
-        </is>
-      </c>
-      <c r="C36" t="inlineStr">
-        <is>
-          <t>Consistent search box placement in the header across all pages</t>
-        </is>
-      </c>
-      <c r="D36" t="inlineStr">
-        <is>
-          <t>DBIM 9(v)</t>
-        </is>
-      </c>
-      <c r="E36" t="inlineStr">
-        <is>
-          <t>Non-compliant</t>
-        </is>
-      </c>
-      <c r="F36" t="inlineStr">
-        <is>
-          <t>Confirmed: only CitizenDashboard.jsx has a header-docked search bar; Uploader/Approver/Admin/Nodal/CSO dashboards each use their own in-page table-filter search box in a different position.</t>
-        </is>
-      </c>
-      <c r="G36" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="H36" t="inlineStr">
-        <is>
-          <t>S</t>
-        </is>
-      </c>
-      <c r="I36" t="inlineStr">
-        <is>
-          <t>Topbar.jsx</t>
-        </is>
-      </c>
-    </row>
-    <row r="37" ht="15.6" customHeight="1">
-      <c r="A37" t="n">
-        <v>36</v>
-      </c>
-      <c r="B37" t="inlineStr">
-        <is>
-          <t>Performance</t>
-        </is>
-      </c>
-      <c r="C37" t="inlineStr">
-        <is>
-          <t>Lazy-load images and media</t>
-        </is>
-      </c>
-      <c r="D37" t="inlineStr">
-        <is>
-          <t>DBIM 10.1.2</t>
-        </is>
-      </c>
-      <c r="E37" t="inlineStr">
-        <is>
-          <t>Missing</t>
-        </is>
-      </c>
-      <c r="F37" t="inlineStr">
-        <is>
-          <t>Confirmed via repo-wide search: zero loading='lazy' attributes found anywhere in src.</t>
-        </is>
-      </c>
-      <c r="G37" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="H37" t="inlineStr">
-        <is>
-          <t>S</t>
-        </is>
-      </c>
-      <c r="I37" t="inlineStr">
-        <is>
-          <t>App-wide</t>
-        </is>
-      </c>
-    </row>
-    <row r="38" ht="15.6" customHeight="1">
-      <c r="A38" t="n">
-        <v>37</v>
-      </c>
-      <c r="B38" t="inlineStr">
-        <is>
-          <t>Performance</t>
-        </is>
-      </c>
-      <c r="C38" t="inlineStr">
-        <is>
-          <t>Image compression/optimization pipeline before publishing</t>
-        </is>
-      </c>
-      <c r="D38" t="inlineStr">
-        <is>
-          <t>DBIM 10.3.2</t>
-        </is>
-      </c>
-      <c r="E38" t="inlineStr">
-        <is>
-          <t>Missing</t>
-        </is>
-      </c>
-      <c r="F38" t="inlineStr">
-        <is>
-          <t>Confirmed: no image-compression/optimization code exists; images are used as-is from src/assets.</t>
-        </is>
-      </c>
-      <c r="G38" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="H38" t="inlineStr">
+      <c r="H43" s="8" t="inlineStr">
         <is>
           <t>M</t>
         </is>
       </c>
-      <c r="I38" t="inlineStr">
-        <is>
-          <t>Upload backend</t>
-        </is>
-      </c>
-    </row>
-    <row r="39" ht="15.6" customHeight="1">
-      <c r="A39" t="n">
-        <v>38</v>
-      </c>
-      <c r="B39" t="inlineStr">
-        <is>
-          <t>Performance</t>
-        </is>
-      </c>
-      <c r="C39" t="inlineStr">
-        <is>
-          <t>Analytics integration (visitor tracking, KPIs, traffic dashboard)</t>
-        </is>
-      </c>
-      <c r="D39" t="inlineStr">
-        <is>
-          <t>DBIM 10.5-10.6</t>
-        </is>
-      </c>
-      <c r="E39" t="inlineStr">
-        <is>
-          <t>Partial</t>
-        </is>
-      </c>
-      <c r="F39" t="inlineStr">
-        <is>
-          <t>CSODashboard.jsx Analytics tab now shows real document KPIs (totals, dept breakdown, status distribution, monthly trend) - but this is content/document analytics, not visitor/traffic tracking as required.</t>
-        </is>
-      </c>
-      <c r="G39" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="H39" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="I39" t="inlineStr">
-        <is>
-          <t>index.html / src/main.jsx</t>
-        </is>
-      </c>
-    </row>
-    <row r="40" ht="15.6" customHeight="1">
-      <c r="A40" t="n">
-        <v>39</v>
-      </c>
-      <c r="B40" t="inlineStr">
-        <is>
-          <t>Forms</t>
-        </is>
-      </c>
-      <c r="C40" t="inlineStr">
-        <is>
-          <t>Mandatory fields marked with * or "Required"; single-column vertical layout; clickable labels; keyboard-friendly</t>
-        </is>
-      </c>
-      <c r="D40" t="inlineStr">
-        <is>
-          <t>DBIM Annexure B</t>
-        </is>
-      </c>
-      <c r="E40" t="inlineStr">
-        <is>
-          <t>Partial</t>
-        </is>
-      </c>
-      <c r="F40" t="inlineStr">
-        <is>
-          <t>Login.jsx is mostly compliant; Add Department / User forms are inconsistent (placeholders instead of labels)</t>
-        </is>
-      </c>
-      <c r="G40" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="H40" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="I40" t="inlineStr">
-        <is>
-          <t>Form components across Admin/Uploader/Nodal dashboards</t>
-        </is>
-      </c>
-    </row>
-    <row r="41" ht="15.6" customHeight="1">
-      <c r="A41" t="n">
-        <v>40</v>
-      </c>
-      <c r="B41" t="inlineStr">
-        <is>
-          <t>Forms</t>
-        </is>
-      </c>
-      <c r="C41" t="inlineStr">
-        <is>
-          <t>Primary action buttons disabled until required fields are valid, with submit-progress feedback</t>
-        </is>
-      </c>
-      <c r="D41" t="inlineStr">
-        <is>
-          <t>DBIM Annexure B(xiv)</t>
-        </is>
-      </c>
-      <c r="E41" t="inlineStr">
-        <is>
-          <t>Partial</t>
-        </is>
-      </c>
-      <c r="F41" t="inlineStr">
-        <is>
-          <t>Some forms already do this (e.g. Add Department drawer disables while creating) - extend the pattern to all forms</t>
-        </is>
-      </c>
-      <c r="G41" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="H41" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="I41" t="inlineStr">
-        <is>
-          <t>Form components app-wide</t>
-        </is>
-      </c>
-    </row>
-    <row r="42" ht="15.6" customHeight="1">
-      <c r="A42" t="n">
-        <v>41</v>
-      </c>
-      <c r="B42" t="inlineStr">
-        <is>
-          <t>Security</t>
-        </is>
-      </c>
-      <c r="C42" t="inlineStr">
-        <is>
-          <t>CAPTCHA on login/OTP/forgot-password forms</t>
-        </is>
-      </c>
-      <c r="D42" t="inlineStr">
-        <is>
-          <t>GIGW security baseline</t>
-        </is>
-      </c>
-      <c r="E42" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="F42" t="inlineStr">
-        <is>
-          <t>No CAPTCHA found on any authentication form</t>
-        </is>
-      </c>
-      <c r="G42" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="H42" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="I42" t="inlineStr">
-        <is>
-          <t>src/pages/Login.jsx, AdminOtpLogin*, ForgotPasswordScreen.jsx</t>
-        </is>
-      </c>
-      <c r="J42" s="1" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-    </row>
-    <row r="43" ht="15.6" customHeight="1">
-      <c r="A43" t="n">
-        <v>42</v>
-      </c>
-      <c r="B43" t="inlineStr">
-        <is>
-          <t>Security</t>
-        </is>
-      </c>
-      <c r="C43" t="inlineStr">
-        <is>
-          <t>Idle/inactivity session timeout (not just reactive 401 logout)</t>
-        </is>
-      </c>
-      <c r="D43" t="inlineStr">
-        <is>
-          <t>GIGW</t>
-        </is>
-      </c>
-      <c r="E43" t="inlineStr">
-        <is>
-          <t>Partial</t>
-        </is>
-      </c>
-      <c r="F43" t="inlineStr">
-        <is>
-          <t>Only a reactive 401-triggered logout exists (services/api.js:17, hooks/useAuth.js:54-55); no idle timer</t>
-        </is>
-      </c>
-      <c r="G43" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="H43" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="I43" t="inlineStr">
+      <c r="I43" s="8" t="inlineStr">
         <is>
           <t>src/hooks/useAuth.js</t>
+        </is>
+      </c>
+      <c r="J43" s="8" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
     </row>

</xml_diff>